<commit_message>
Move benchmarks to daily-change sheet; add 锐进1号 - CSI500 excess + daily chart
Sheet "今年以来收益率" no longer carries benchmark rows. Sheet
"单日单位净值变动" now appends three rows at the bottom:
  - 沪深300 (单日)
  - 中证500 (单日)
  - 锐进1号 - 中证500 超额  (daily 锐进1号 NAV change minus CSI 500 daily)

Daily benchmark % comes from the cached close series; previous trading
day is the most recent date < target in the cache.

New chart <stem>_daily_chart.png plots every product's daily NAV change,
the two benchmark daily series, and the excess line on one canvas.

https://claude.ai/code/session_014VmLcPuADdRYg34QDm2fTF
</commit_message>
<xml_diff>
--- a/output/20260410_20260514_table.xlsx
+++ b/output/20260410_20260514_table.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +41,12 @@
       <b val="1"/>
       <i val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -100,13 +109,19 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -477,7 +492,7 @@
   <dimension ref="A1:W8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1141,10 +1156,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W10"/>
+  <dimension ref="A1:W8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1797,152 +1812,6 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>沪深300 (自2026-02-27起)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>-0.01572637507600072</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>-0.01369075232533347</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>-0.001987667553685626</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>-0.005392146883265597</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>0.005511090207164507</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0.003826374674781916</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>0.009933879781989195</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>0.01217456990885913</v>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>0.01888914662654946</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>0.01606581890058459</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>0.01246578256587231</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>0.01280078963252376</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>0.01009657505851277</v>
-      </c>
-      <c r="O9" s="6" t="n">
-        <v>0.02116480010420661</v>
-      </c>
-      <c r="P9" s="6" t="n">
-        <v>0.02051947472437381</v>
-      </c>
-      <c r="Q9" s="6" t="n">
-        <v>0.03533406420251973</v>
-      </c>
-      <c r="R9" s="6" t="n">
-        <v>0.0403050587383232</v>
-      </c>
-      <c r="S9" s="6" t="n">
-        <v>0.03423421526245154</v>
-      </c>
-      <c r="T9" s="6" t="n">
-        <v>0.05120097199388898</v>
-      </c>
-      <c r="U9" s="6" t="n">
-        <v>0.05039639035564322</v>
-      </c>
-      <c r="V9" s="6" t="n">
-        <v>0.06107331033451057</v>
-      </c>
-      <c r="W9" s="6" t="n">
-        <v>0.04329558218426438</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>中证500 (自2026-02-27起)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>-0.07958533872972633</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>-0.07977793670537096</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>-0.06581796744851681</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>-0.07095646203570638</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>-0.05524877817916216</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>-0.05130899694602396</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>-0.04255125192553228</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>-0.04482600079138874</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>-0.03260046431172566</v>
-      </c>
-      <c r="K10" s="6" t="n">
-        <v>-0.0419524611696391</v>
-      </c>
-      <c r="L10" s="6" t="n">
-        <v>-0.04741892437726429</v>
-      </c>
-      <c r="M10" s="6" t="n">
-        <v>-0.04150877900171123</v>
-      </c>
-      <c r="N10" s="6" t="n">
-        <v>-0.05249079041315283</v>
-      </c>
-      <c r="O10" s="6" t="n">
-        <v>-0.03649944147626506</v>
-      </c>
-      <c r="P10" s="6" t="n">
-        <v>-0.03568100402447321</v>
-      </c>
-      <c r="Q10" s="6" t="n">
-        <v>-0.008085788746746174</v>
-      </c>
-      <c r="R10" s="6" t="n">
-        <v>0.00442903737635352</v>
-      </c>
-      <c r="S10" s="6" t="n">
-        <v>0.004125518858726802</v>
-      </c>
-      <c r="T10" s="6" t="n">
-        <v>0.02093806555660424</v>
-      </c>
-      <c r="U10" s="6" t="n">
-        <v>0.01472882508778737</v>
-      </c>
-      <c r="V10" s="6" t="n">
-        <v>0.03000406435317866</v>
-      </c>
-      <c r="W10" s="6" t="n">
-        <v>0.001352101079797112</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1954,10 +1823,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -2105,70 +1974,70 @@
           <t>瑞享1号</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="D2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="E2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="G2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="H2" s="7" t="n">
+      <c r="H2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="I2" s="7" t="n">
+      <c r="I2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="J2" s="7" t="n">
+      <c r="J2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="K2" s="7" t="n">
+      <c r="K2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="L2" s="7" t="n">
+      <c r="L2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="M2" s="7" t="n">
+      <c r="M2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="N2" s="7" t="n">
+      <c r="N2" s="5" t="n">
         <v>4e-05</v>
       </c>
-      <c r="O2" s="7" t="n">
+      <c r="O2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="P2" s="7" t="n">
+      <c r="P2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="Q2" s="7" t="n">
+      <c r="Q2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="R2" s="7" t="n">
+      <c r="R2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="S2" s="7" t="n">
+      <c r="S2" s="5" t="n">
         <v>4e-05</v>
       </c>
-      <c r="T2" s="7" t="n">
+      <c r="T2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="U2" s="7" t="n">
+      <c r="U2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="V2" s="7" t="n">
+      <c r="V2" s="5" t="n">
         <v>5e-05</v>
       </c>
-      <c r="W2" s="7" t="n">
+      <c r="W2" s="5" t="n">
         <v>5e-05</v>
       </c>
     </row>
@@ -2178,70 +2047,70 @@
           <t>瑞享3号</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="5" t="n">
         <v>0.0307</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="5" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="5" t="n">
         <v>-0.0128</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="E3" s="5" t="n">
         <v>-0.0118</v>
       </c>
-      <c r="F3" s="7" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.0048</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="5" t="n">
         <v>-0.0034</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="H3" s="5" t="n">
         <v>0.0541</v>
       </c>
-      <c r="I3" s="7" t="n">
+      <c r="I3" s="5" t="n">
         <v>0.0495</v>
       </c>
-      <c r="J3" s="7" t="n">
+      <c r="J3" s="5" t="n">
         <v>0.0147</v>
       </c>
-      <c r="K3" s="7" t="n">
+      <c r="K3" s="5" t="n">
         <v>-0.0392</v>
       </c>
-      <c r="L3" s="7" t="n">
+      <c r="L3" s="5" t="n">
         <v>-0.0273</v>
       </c>
-      <c r="M3" s="7" t="n">
+      <c r="M3" s="5" t="n">
         <v>-0.0113</v>
       </c>
-      <c r="N3" s="7" t="n">
+      <c r="N3" s="5" t="n">
         <v>0.0004</v>
       </c>
-      <c r="O3" s="7" t="n">
+      <c r="O3" s="5" t="n">
         <v>-0.0244</v>
       </c>
-      <c r="P3" s="7" t="n">
+      <c r="P3" s="5" t="n">
         <v>0.0349</v>
       </c>
-      <c r="Q3" s="7" t="n">
+      <c r="Q3" s="5" t="n">
         <v>0.0129</v>
       </c>
-      <c r="R3" s="7" t="n">
+      <c r="R3" s="5" t="n">
         <v>0.0226</v>
       </c>
-      <c r="S3" s="7" t="n">
+      <c r="S3" s="5" t="n">
         <v>0.0063</v>
       </c>
-      <c r="T3" s="7" t="n">
+      <c r="T3" s="5" t="n">
         <v>-0.0185</v>
       </c>
-      <c r="U3" s="7" t="n">
+      <c r="U3" s="5" t="n">
         <v>-0.0038</v>
       </c>
-      <c r="V3" s="7" t="n">
+      <c r="V3" s="5" t="n">
         <v>0.0008</v>
       </c>
-      <c r="W3" s="7" t="n">
+      <c r="W3" s="5" t="n">
         <v>-0.0375</v>
       </c>
     </row>
@@ -2251,70 +2120,70 @@
           <t>配置1号</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="5" t="n">
         <v>0.0052</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C4" s="5" t="n">
         <v>0.0014</v>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="5" t="n">
         <v>0.0039</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F4" s="7" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.004099999999999999</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="5" t="n">
         <v>0.0011</v>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="H4" s="5" t="n">
         <v>-0.0028</v>
       </c>
-      <c r="I4" s="7" t="n">
+      <c r="I4" s="5" t="n">
         <v>-0.0014</v>
       </c>
-      <c r="J4" s="7" t="n">
+      <c r="J4" s="5" t="n">
         <v>0.0048</v>
       </c>
-      <c r="K4" s="7" t="n">
+      <c r="K4" s="5" t="n">
         <v>-0.006500000000000001</v>
       </c>
-      <c r="L4" s="7" t="n">
+      <c r="L4" s="5" t="n">
         <v>0.0019</v>
       </c>
-      <c r="M4" s="7" t="n">
+      <c r="M4" s="5" t="n">
         <v>0.0018</v>
       </c>
-      <c r="N4" s="7" t="n">
+      <c r="N4" s="5" t="n">
         <v>0.001</v>
       </c>
-      <c r="O4" s="7" t="n">
+      <c r="O4" s="5" t="n">
         <v>0.0107</v>
       </c>
-      <c r="P4" s="7" t="n">
+      <c r="P4" s="5" t="n">
         <v>0.0016</v>
       </c>
-      <c r="Q4" s="7" t="n">
+      <c r="Q4" s="5" t="n">
         <v>0.0064</v>
       </c>
-      <c r="R4" s="7" t="n">
+      <c r="R4" s="5" t="n">
         <v>0.0003</v>
       </c>
-      <c r="S4" s="7" t="n">
+      <c r="S4" s="5" t="n">
         <v>-0.0049</v>
       </c>
-      <c r="T4" s="7" t="n">
+      <c r="T4" s="5" t="n">
         <v>0.012</v>
       </c>
-      <c r="U4" s="7" t="n">
+      <c r="U4" s="5" t="n">
         <v>0.0004</v>
       </c>
-      <c r="V4" s="7" t="n">
+      <c r="V4" s="5" t="n">
         <v>0.009899999999999999</v>
       </c>
-      <c r="W4" s="7" t="n">
+      <c r="W4" s="5" t="n">
         <v>-0.0131</v>
       </c>
     </row>
@@ -2324,70 +2193,70 @@
           <t>瑞臻1号</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="5" t="n">
         <v>0.0193</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="5" t="n">
         <v>0.0063</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="5" t="n">
         <v>-0.0138</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="5" t="n">
         <v>-0.0275</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="5" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="5" t="n">
         <v>-0.008199999999999999</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="5" t="n">
         <v>0.0336</v>
       </c>
-      <c r="I5" s="7" t="n">
+      <c r="I5" s="5" t="n">
         <v>0.05400000000000001</v>
       </c>
-      <c r="J5" s="7" t="n">
+      <c r="J5" s="5" t="n">
         <v>-0.0075</v>
       </c>
-      <c r="K5" s="7" t="n">
+      <c r="K5" s="5" t="n">
         <v>-0.0199</v>
       </c>
-      <c r="L5" s="7" t="n">
+      <c r="L5" s="5" t="n">
         <v>-0.0104</v>
       </c>
-      <c r="M5" s="7" t="n">
+      <c r="M5" s="5" t="n">
         <v>-0.0125</v>
       </c>
-      <c r="N5" s="7" t="n">
+      <c r="N5" s="5" t="n">
         <v>-0.0066</v>
       </c>
-      <c r="O5" s="7" t="n">
+      <c r="O5" s="5" t="n">
         <v>-0.0068</v>
       </c>
-      <c r="P5" s="7" t="n">
+      <c r="P5" s="5" t="n">
         <v>0.005500000000000001</v>
       </c>
-      <c r="Q5" s="7" t="n">
+      <c r="Q5" s="5" t="n">
         <v>0.0009</v>
       </c>
-      <c r="R5" s="7" t="n">
+      <c r="R5" s="5" t="n">
         <v>-0.005600000000000001</v>
       </c>
-      <c r="S5" s="7" t="n">
+      <c r="S5" s="5" t="n">
         <v>0.0222</v>
       </c>
-      <c r="T5" s="7" t="n">
+      <c r="T5" s="5" t="n">
         <v>0.0025</v>
       </c>
-      <c r="U5" s="7" t="n">
+      <c r="U5" s="5" t="n">
         <v>-0.0226</v>
       </c>
-      <c r="V5" s="7" t="n">
+      <c r="V5" s="5" t="n">
         <v>0.0012</v>
       </c>
-      <c r="W5" s="7" t="n">
+      <c r="W5" s="5" t="n">
         <v>-0.03700000000000001</v>
       </c>
     </row>
@@ -2397,70 +2266,70 @@
           <t>鑫盛1号</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="5" t="n">
         <v>0.0068</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="5" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="5" t="n">
         <v>0.0051</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="5" t="n">
         <v>0.0011</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.004699999999999999</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="5" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="5" t="n">
         <v>-0.002</v>
       </c>
-      <c r="I6" s="7" t="n">
+      <c r="I6" s="5" t="n">
         <v>-0.0011</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="5" t="n">
         <v>0.0052</v>
       </c>
-      <c r="K6" s="7" t="n">
+      <c r="K6" s="5" t="n">
         <v>-0.006500000000000001</v>
       </c>
-      <c r="L6" s="7" t="n">
+      <c r="L6" s="5" t="n">
         <v>0.0019</v>
       </c>
-      <c r="M6" s="7" t="n">
+      <c r="M6" s="5" t="n">
         <v>0.0017</v>
       </c>
-      <c r="N6" s="7" t="n">
+      <c r="N6" s="5" t="n">
         <v>0.0016</v>
       </c>
-      <c r="O6" s="7" t="n">
+      <c r="O6" s="5" t="n">
         <v>0.0109</v>
       </c>
-      <c r="P6" s="7" t="n">
+      <c r="P6" s="5" t="n">
         <v>0.0019</v>
       </c>
-      <c r="Q6" s="7" t="n">
+      <c r="Q6" s="5" t="n">
         <v>0.008</v>
       </c>
-      <c r="R6" s="7" t="n">
+      <c r="R6" s="5" t="n">
         <v>0.0008</v>
       </c>
-      <c r="S6" s="7" t="n">
+      <c r="S6" s="5" t="n">
         <v>-0.0052</v>
       </c>
-      <c r="T6" s="7" t="n">
+      <c r="T6" s="5" t="n">
         <v>0.012</v>
       </c>
-      <c r="U6" s="7" t="n">
+      <c r="U6" s="5" t="n">
         <v>0.0011</v>
       </c>
-      <c r="V6" s="7" t="n">
+      <c r="V6" s="5" t="n">
         <v>0.0102</v>
       </c>
-      <c r="W6" s="7" t="n">
+      <c r="W6" s="5" t="n">
         <v>-0.0145</v>
       </c>
     </row>
@@ -2470,70 +2339,70 @@
           <t>领航1号</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="5" t="n">
         <v>0.0185</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="5" t="n">
         <v>0.0025</v>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="5" t="n">
         <v>0.0165</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="5" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.0233</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="5" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="5" t="n">
         <v>0.004</v>
       </c>
-      <c r="I7" s="7" t="n">
+      <c r="I7" s="5" t="n">
         <v>0.0005</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="J7" s="5" t="n">
         <v>0.014</v>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K7" s="5" t="n">
         <v>-0.0197</v>
       </c>
-      <c r="L7" s="7" t="n">
+      <c r="L7" s="5" t="n">
         <v>0.0027</v>
       </c>
-      <c r="M7" s="7" t="n">
+      <c r="M7" s="5" t="n">
         <v>0.0072</v>
       </c>
-      <c r="N7" s="7" t="n">
+      <c r="N7" s="5" t="n">
         <v>-0.0071</v>
       </c>
-      <c r="O7" s="7" t="n">
+      <c r="O7" s="5" t="n">
         <v>0.0306</v>
       </c>
-      <c r="P7" s="7" t="n">
+      <c r="P7" s="5" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="Q7" s="7" t="n">
+      <c r="Q7" s="5" t="n">
         <v>0.04099999999999999</v>
       </c>
-      <c r="R7" s="7" t="n">
+      <c r="R7" s="5" t="n">
         <v>0.0137</v>
       </c>
-      <c r="S7" s="7" t="n">
+      <c r="S7" s="5" t="n">
         <v>-0.009599999999999999</v>
       </c>
-      <c r="T7" s="7" t="n">
+      <c r="T7" s="5" t="n">
         <v>0.0263</v>
       </c>
-      <c r="U7" s="7" t="n">
+      <c r="U7" s="5" t="n">
         <v>-0.0058</v>
       </c>
-      <c r="V7" s="7" t="n">
+      <c r="V7" s="5" t="n">
         <v>0.0186</v>
       </c>
-      <c r="W7" s="7" t="n">
+      <c r="W7" s="5" t="n">
         <v>-0.03</v>
       </c>
     </row>
@@ -2543,71 +2412,290 @@
           <t>锐进1号</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="5" t="n">
         <v>0.0039</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="5" t="n">
         <v>0.0014</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="5" t="n">
         <v>0.0025</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.0022</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="5" t="n">
         <v>0.0015</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="5" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="I8" s="7" t="n">
+      <c r="I8" s="5" t="n">
         <v>-0.0013</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="5" t="n">
         <v>0.0031</v>
       </c>
-      <c r="K8" s="7" t="n">
+      <c r="K8" s="5" t="n">
         <v>-0.005699999999999999</v>
       </c>
-      <c r="L8" s="7" t="n">
+      <c r="L8" s="5" t="n">
         <v>0.0022</v>
       </c>
-      <c r="M8" s="7" t="n">
+      <c r="M8" s="5" t="n">
         <v>0.0018</v>
       </c>
-      <c r="N8" s="7" t="n">
+      <c r="N8" s="5" t="n">
         <v>0.0021</v>
       </c>
-      <c r="O8" s="7" t="n">
+      <c r="O8" s="5" t="n">
         <v>0.008</v>
       </c>
-      <c r="P8" s="7" t="n">
+      <c r="P8" s="5" t="n">
         <v>0.002</v>
       </c>
-      <c r="Q8" s="7" t="n">
+      <c r="Q8" s="5" t="n">
         <v>0.0034</v>
       </c>
-      <c r="R8" s="7" t="n">
+      <c r="R8" s="5" t="n">
         <v>-0.0009</v>
       </c>
-      <c r="S8" s="7" t="n">
+      <c r="S8" s="5" t="n">
         <v>-0.0048</v>
       </c>
-      <c r="T8" s="7" t="n">
+      <c r="T8" s="5" t="n">
         <v>0.0103</v>
       </c>
-      <c r="U8" s="7" t="n">
+      <c r="U8" s="5" t="n">
         <v>0.0012</v>
       </c>
-      <c r="V8" s="7" t="n">
+      <c r="V8" s="5" t="n">
         <v>0.0083</v>
       </c>
-      <c r="W8" s="7" t="n">
+      <c r="W8" s="5" t="n">
         <v>-0.0116</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>沪深300 (单日)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.01540480813500227</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>0.002068147209394571</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0.0118655328430096</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>-0.003411259779961792</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>0.01096234767930233</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>-0.001675481801036615</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>0.006084224584342067</v>
+      </c>
+      <c r="I9" s="7" t="n">
+        <v>0.002218650321299876</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0.006633812898791696</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>-0.002770986162049777</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>-0.003543113317804182</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>0.0003308823591079226</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>-0.00267003600480225</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>0.01095759090664442</v>
+      </c>
+      <c r="P9" s="7" t="n">
+        <v>-0.0006319502785122833</v>
+      </c>
+      <c r="Q9" s="7" t="n">
+        <v>0.01451671412948499</v>
+      </c>
+      <c r="R9" s="7" t="n">
+        <v>0.004801343554394154</v>
+      </c>
+      <c r="S9" s="7" t="n">
+        <v>-0.005835637753443541</v>
+      </c>
+      <c r="T9" s="7" t="n">
+        <v>0.01640513964927362</v>
+      </c>
+      <c r="U9" s="7" t="n">
+        <v>-0.0007653927837601216</v>
+      </c>
+      <c r="V9" s="7" t="n">
+        <v>0.01016465791095528</v>
+      </c>
+      <c r="W9" s="7" t="n">
+        <v>-0.0167544767897721</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>中证500 (单日)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.008954929403036351</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>-0.000209251312206216</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>0.0151702179437797</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>-0.005500528171319097</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>0.01690737109152349</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>0.004170178500055284</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>0.009231398835130933</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>-0.002375844002544493</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>0.01279927687499061</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>-0.00966715045119367</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>-0.005705837117747784</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.006204348928189013</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>-0.01145760250156867</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>0.01687724908115738</v>
+      </c>
+      <c r="P10" s="7" t="n">
+        <v>0.0008494415955978729</v>
+      </c>
+      <c r="Q10" s="7" t="n">
+        <v>0.02861627261610781</v>
+      </c>
+      <c r="R10" s="7" t="n">
+        <v>0.01261684325228851</v>
+      </c>
+      <c r="S10" s="7" t="n">
+        <v>-0.0003021801504460005</v>
+      </c>
+      <c r="T10" s="7" t="n">
+        <v>0.01674347119171547</v>
+      </c>
+      <c r="U10" s="7" t="n">
+        <v>-0.006081897304349864</v>
+      </c>
+      <c r="V10" s="7" t="n">
+        <v>0.01505351862264265</v>
+      </c>
+      <c r="W10" s="7" t="n">
+        <v>-0.02781733030478321</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>锐进1号 - 中证500 超额</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>-0.005054929403036351</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0.001609251312206216</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-0.0126702179437797</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0.005600528171319097</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>-0.01470737109152349</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>-0.002670178500055284</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>-0.01243139883513093</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0.001075844002544494</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>-0.009699276874990614</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0.003967150451193671</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>0.007905837117747784</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>-0.004404348928189013</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>0.01355760250156867</v>
+      </c>
+      <c r="O11" s="9" t="n">
+        <v>-0.008877249081157383</v>
+      </c>
+      <c r="P11" s="9" t="n">
+        <v>0.001150558404402127</v>
+      </c>
+      <c r="Q11" s="9" t="n">
+        <v>-0.02521627261610781</v>
+      </c>
+      <c r="R11" s="9" t="n">
+        <v>-0.01351684325228851</v>
+      </c>
+      <c r="S11" s="9" t="n">
+        <v>-0.004497819849553999</v>
+      </c>
+      <c r="T11" s="9" t="n">
+        <v>-0.006443471191715467</v>
+      </c>
+      <c r="U11" s="9" t="n">
+        <v>0.007281897304349864</v>
+      </c>
+      <c r="V11" s="9" t="n">
+        <v>-0.00675351862264265</v>
+      </c>
+      <c r="W11" s="9" t="n">
+        <v>0.01621733030478321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Switch daily excess row/line from 锐进1号 to 领航1号 vs CSI500
https://claude.ai/code/session_014VmLcPuADdRYg34QDm2fTF
</commit_message>
<xml_diff>
--- a/output/20260410_20260514_table.xlsx
+++ b/output/20260410_20260514_table.xlsx
@@ -2628,74 +2628,74 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>锐进1号 - 中证500 超额</t>
+          <t>领航1号 - 中证500 超额</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>-0.005054929403036351</v>
+        <v>0.00954507059696365</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>0.001609251312206216</v>
+        <v>0.002709251312206216</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>-0.0126702179437797</v>
+        <v>0.001329782056220299</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.005600528171319097</v>
+        <v>0.006200528171319097</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>-0.01470737109152349</v>
+        <v>0.006392628908476512</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>-0.002670178500055284</v>
+        <v>-0.004870178500055284</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>-0.01243139883513093</v>
+        <v>-0.005231398835130932</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.001075844002544494</v>
+        <v>0.002875844002544493</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>-0.009699276874990614</v>
+        <v>0.001200723125009384</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>0.003967150451193671</v>
+        <v>-0.01003284954880633</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.007905837117747784</v>
+        <v>0.008405837117747785</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>-0.004404348928189013</v>
+        <v>0.0009956510718109868</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>0.01355760250156867</v>
+        <v>0.004357602501568667</v>
       </c>
       <c r="O11" s="9" t="n">
-        <v>-0.008877249081157383</v>
+        <v>0.01372275091884262</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>0.001150558404402127</v>
+        <v>-0.0001494415955978729</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.02521627261610781</v>
+        <v>0.01238372738389219</v>
       </c>
       <c r="R11" s="9" t="n">
-        <v>-0.01351684325228851</v>
+        <v>0.001083156747711493</v>
       </c>
       <c r="S11" s="9" t="n">
-        <v>-0.004497819849553999</v>
+        <v>-0.009297819849553999</v>
       </c>
       <c r="T11" s="9" t="n">
-        <v>-0.006443471191715467</v>
+        <v>0.009556528808284533</v>
       </c>
       <c r="U11" s="9" t="n">
-        <v>0.007281897304349864</v>
+        <v>0.000281897304349864</v>
       </c>
       <c r="V11" s="9" t="n">
-        <v>-0.00675351862264265</v>
+        <v>0.003546481377357351</v>
       </c>
       <c r="W11" s="9" t="n">
-        <v>0.01621733030478321</v>
+        <v>-0.002182669695216788</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add CSI 300/500 closing points + cumulative excess to NAV sheet; nav chart
基金单位净值 sheet now appends three rows: 沪深300 (收盘点位),
中证500 (收盘点位), and 领航1号 - 中证500 累计超额 (region-return
difference in percentage points, first date = 0).

New <stem>_nav_chart.png: funds and index points rebased to 100 at the
first date (different scales otherwise), with the cumulative excess on a
secondary axis.

https://claude.ai/code/session_014VmLcPuADdRYg34QDm2fTF
</commit_message>
<xml_diff>
--- a/output/20260410_20260514_table.xlsx
+++ b/output/20260410_20260514_table.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -106,20 +106,26 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -489,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1149,225 @@
       </c>
       <c r="W8" s="3" t="n">
         <v>1.03</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>沪深300 (收盘点位)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>4636.5655</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>4646.1546</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>4701.2837</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>4685.2464</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>4736.6077</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>4728.6716</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>4757.4419</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>4767.997</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>4799.627</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>4786.3273</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>4769.3688</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>4770.9469</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>4758.2083</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>4810.3468</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>4807.3069</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>4877.0932</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>4900.5098</v>
+      </c>
+      <c r="S9" s="5" t="n">
+        <v>4871.9122</v>
+      </c>
+      <c r="T9" s="5" t="n">
+        <v>4951.8366</v>
+      </c>
+      <c r="U9" s="5" t="n">
+        <v>4948.0465</v>
+      </c>
+      <c r="V9" s="5" t="n">
+        <v>4998.3417</v>
+      </c>
+      <c r="W9" s="5" t="n">
+        <v>4914.5971</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>中证500 (收盘点位)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>7969.3646</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>7967.697</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>8088.5687</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>8044.0773</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>8180.0815</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>8214.1939</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>8290.0224</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>8270.3266</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>8376.1808</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>8295.207</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>8247.875899999999</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>8299.0486</v>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>8203.9614</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>8342.421700000001</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>8349.508099999999</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>8588.439899999999</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>8696.7989</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>8694.170899999999</v>
+      </c>
+      <c r="T10" s="5" t="n">
+        <v>8839.7415</v>
+      </c>
+      <c r="U10" s="5" t="n">
+        <v>8785.9791</v>
+      </c>
+      <c r="V10" s="5" t="n">
+        <v>8918.239</v>
+      </c>
+      <c r="W10" s="5" t="n">
+        <v>8670.1574</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>领航1号 - 中证500 累计超额</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>0.002564039381279914</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>0.003978628478572777</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>0.01024824559432114</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>0.01692648112621087</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>0.01195922630920832</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>0.006466989783670885</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>0.009429009822418566</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>0.01076567921138882</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>2.756948569748729e-05</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>0.008812069359058539</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0.009847721329049319</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>0.01432248357702504</v>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>0.02893428464983949</v>
+      </c>
+      <c r="P11" s="7" t="n">
+        <v>0.02883000886178766</v>
+      </c>
+      <c r="Q11" s="7" t="n">
+        <v>0.04270665056181477</v>
+      </c>
+      <c r="R11" s="7" t="n">
+        <v>0.04451394570507161</v>
+      </c>
+      <c r="S11" s="7" t="n">
+        <v>0.03395281368752312</v>
+      </c>
+      <c r="T11" s="7" t="n">
+        <v>0.04512139022337847</v>
+      </c>
+      <c r="U11" s="7" t="n">
+        <v>0.04519562450781467</v>
+      </c>
+      <c r="V11" s="7" t="n">
+        <v>0.04998890867505268</v>
+      </c>
+      <c r="W11" s="7" t="n">
+        <v>0.0460908438797849</v>
       </c>
     </row>
   </sheetData>
@@ -1307,70 +1532,70 @@
           <t>瑞享1号</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="8" t="n">
         <v>0.0062</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="8" t="n">
         <v>0.0064</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="8" t="n">
         <v>0.0064</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="8" t="n">
         <v>0.006500000000000001</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="8" t="n">
         <v>0.006500000000000001</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="8" t="n">
         <v>0.0066</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="8" t="n">
         <v>0.0067</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="8" t="n">
         <v>0.0067</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="8" t="n">
         <v>0.0068</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="K2" s="8" t="n">
         <v>0.0068</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="L2" s="8" t="n">
         <v>0.0069</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="M2" s="8" t="n">
         <v>0.006999999999999999</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N2" s="8" t="n">
         <v>0.0071</v>
       </c>
-      <c r="O2" s="4" t="n">
+      <c r="O2" s="8" t="n">
         <v>0.0071</v>
       </c>
-      <c r="P2" s="4" t="n">
+      <c r="P2" s="8" t="n">
         <v>0.0072</v>
       </c>
-      <c r="Q2" s="4" t="n">
+      <c r="Q2" s="8" t="n">
         <v>0.0075</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="R2" s="8" t="n">
         <v>0.0075</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="S2" s="8" t="n">
         <v>0.0076</v>
       </c>
-      <c r="T2" s="4" t="n">
+      <c r="T2" s="8" t="n">
         <v>0.0077</v>
       </c>
-      <c r="U2" s="4" t="n">
+      <c r="U2" s="8" t="n">
         <v>0.0077</v>
       </c>
-      <c r="V2" s="4" t="n">
+      <c r="V2" s="8" t="n">
         <v>0.007800000000000001</v>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="W2" s="8" t="n">
         <v>0.007800000000000001</v>
       </c>
     </row>
@@ -1380,70 +1605,70 @@
           <t>瑞享3号</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="8" t="n">
         <v>-0.163</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="8" t="n">
         <v>-0.1637</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="8" t="n">
         <v>-0.1743</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="8" t="n">
         <v>-0.1841</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="8" t="n">
         <v>-0.1802</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="8" t="n">
         <v>-0.183</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="8" t="n">
         <v>-0.1389</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="8" t="n">
         <v>-0.09619999999999999</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="8" t="n">
         <v>-0.083</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="8" t="n">
         <v>-0.1189</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="8" t="n">
         <v>-0.1429</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="M3" s="8" t="n">
         <v>-0.1527</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="N3" s="8" t="n">
         <v>-0.1523</v>
       </c>
-      <c r="O3" s="4" t="n">
+      <c r="O3" s="8" t="n">
         <v>-0.173</v>
       </c>
-      <c r="P3" s="4" t="n">
+      <c r="P3" s="8" t="n">
         <v>-0.1441</v>
       </c>
-      <c r="Q3" s="4" t="n">
+      <c r="Q3" s="8" t="n">
         <v>-0.1333</v>
       </c>
-      <c r="R3" s="4" t="n">
+      <c r="R3" s="8" t="n">
         <v>-0.1136</v>
       </c>
-      <c r="S3" s="4" t="n">
+      <c r="S3" s="8" t="n">
         <v>-0.1081</v>
       </c>
-      <c r="T3" s="4" t="n">
+      <c r="T3" s="8" t="n">
         <v>-0.1246</v>
       </c>
-      <c r="U3" s="4" t="n">
+      <c r="U3" s="8" t="n">
         <v>-0.1279</v>
       </c>
-      <c r="V3" s="4" t="n">
+      <c r="V3" s="8" t="n">
         <v>-0.1272</v>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="W3" s="8" t="n">
         <v>-0.1599</v>
       </c>
     </row>
@@ -1453,70 +1678,70 @@
           <t>配置1号</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="8" t="n">
         <v>0.0104</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="8" t="n">
         <v>0.0117</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="8" t="n">
         <v>0.0156</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="8" t="n">
         <v>0.0159</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="8" t="n">
         <v>0.02</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="8" t="n">
         <v>0.0212</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="8" t="n">
         <v>0.0183</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="8" t="n">
         <v>0.0169</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="8" t="n">
         <v>0.0218</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="8" t="n">
         <v>0.0151</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="8" t="n">
         <v>0.0171</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="M4" s="8" t="n">
         <v>0.0188</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="N4" s="8" t="n">
         <v>0.0198</v>
       </c>
-      <c r="O4" s="4" t="n">
+      <c r="O4" s="8" t="n">
         <v>0.0307</v>
       </c>
-      <c r="P4" s="4" t="n">
+      <c r="P4" s="8" t="n">
         <v>0.0323</v>
       </c>
-      <c r="Q4" s="4" t="n">
+      <c r="Q4" s="8" t="n">
         <v>0.0388</v>
       </c>
-      <c r="R4" s="4" t="n">
+      <c r="R4" s="8" t="n">
         <v>0.039</v>
       </c>
-      <c r="S4" s="4" t="n">
+      <c r="S4" s="8" t="n">
         <v>0.0339</v>
       </c>
-      <c r="T4" s="4" t="n">
+      <c r="T4" s="8" t="n">
         <v>0.0463</v>
       </c>
-      <c r="U4" s="4" t="n">
+      <c r="U4" s="8" t="n">
         <v>0.0467</v>
       </c>
-      <c r="V4" s="4" t="n">
+      <c r="V4" s="8" t="n">
         <v>0.057</v>
       </c>
-      <c r="W4" s="4" t="n">
+      <c r="W4" s="8" t="n">
         <v>0.0432</v>
       </c>
     </row>
@@ -1526,70 +1751,70 @@
           <t>瑞臻1号</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="8" t="n">
         <v>-0.09570000000000001</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="8" t="n">
         <v>-0.0901</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="8" t="n">
         <v>-0.1026</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="8" t="n">
         <v>-0.1273</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="8" t="n">
         <v>-0.1301</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="8" t="n">
         <v>-0.1372</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="8" t="n">
         <v>-0.1083</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="8" t="n">
         <v>-0.0604</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="8" t="n">
         <v>-0.0673</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="8" t="n">
         <v>-0.0858</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" s="8" t="n">
         <v>-0.0953</v>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M5" s="8" t="n">
         <v>-0.1067</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="N5" s="8" t="n">
         <v>-0.1126</v>
       </c>
-      <c r="O5" s="4" t="n">
+      <c r="O5" s="8" t="n">
         <v>-0.1186</v>
       </c>
-      <c r="P5" s="4" t="n">
+      <c r="P5" s="8" t="n">
         <v>-0.1137</v>
       </c>
-      <c r="Q5" s="4" t="n">
+      <c r="Q5" s="8" t="n">
         <v>-0.1131</v>
       </c>
-      <c r="R5" s="4" t="n">
+      <c r="R5" s="8" t="n">
         <v>-0.1181</v>
       </c>
-      <c r="S5" s="4" t="n">
+      <c r="S5" s="8" t="n">
         <v>-0.09859999999999999</v>
       </c>
-      <c r="T5" s="4" t="n">
+      <c r="T5" s="8" t="n">
         <v>-0.0964</v>
       </c>
-      <c r="U5" s="4" t="n">
+      <c r="U5" s="8" t="n">
         <v>-0.1168</v>
       </c>
-      <c r="V5" s="4" t="n">
+      <c r="V5" s="8" t="n">
         <v>-0.1158</v>
       </c>
-      <c r="W5" s="4" t="n">
+      <c r="W5" s="8" t="n">
         <v>-0.1485</v>
       </c>
     </row>
@@ -1599,70 +1824,70 @@
           <t>鑫盛1号</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.1378</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="8" t="n">
         <v>0.1385</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="8" t="n">
         <v>0.1443</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="8" t="n">
         <v>0.1455</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="8" t="n">
         <v>0.1509</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="8" t="n">
         <v>0.1517</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="8" t="n">
         <v>0.1493</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="8" t="n">
         <v>0.148</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="8" t="n">
         <v>0.154</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="K6" s="8" t="n">
         <v>0.1465</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L6" s="8" t="n">
         <v>0.1486</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="M6" s="8" t="n">
         <v>0.1506</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N6" s="8" t="n">
         <v>0.1524</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="O6" s="8" t="n">
         <v>0.1649</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="P6" s="8" t="n">
         <v>0.1671</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="Q6" s="8" t="n">
         <v>0.1764</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="R6" s="8" t="n">
         <v>0.1774</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="S6" s="8" t="n">
         <v>0.1712</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="T6" s="8" t="n">
         <v>0.1853</v>
       </c>
-      <c r="U6" s="4" t="n">
+      <c r="U6" s="8" t="n">
         <v>0.1867</v>
       </c>
-      <c r="V6" s="4" t="n">
+      <c r="V6" s="8" t="n">
         <v>0.1987</v>
       </c>
-      <c r="W6" s="4" t="n">
+      <c r="W6" s="8" t="n">
         <v>0.1813</v>
       </c>
     </row>
@@ -1672,70 +1897,70 @@
           <t>领航1号</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="8" t="n">
         <v>0.0191</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="8" t="n">
         <v>0.0216</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="8" t="n">
         <v>0.0385</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="8" t="n">
         <v>0.0392</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="8" t="n">
         <v>0.0633</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="8" t="n">
         <v>0.0626</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="8" t="n">
         <v>0.0668</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="8" t="n">
         <v>0.0673</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="8" t="n">
         <v>0.08220000000000001</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="K7" s="8" t="n">
         <v>0.0609</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="L7" s="8" t="n">
         <v>0.0638</v>
       </c>
-      <c r="M7" s="4" t="n">
+      <c r="M7" s="8" t="n">
         <v>0.07139999999999999</v>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="N7" s="8" t="n">
         <v>0.0638</v>
       </c>
-      <c r="O7" s="4" t="n">
+      <c r="O7" s="8" t="n">
         <v>0.0964</v>
       </c>
-      <c r="P7" s="4" t="n">
+      <c r="P7" s="8" t="n">
         <v>0.09710000000000001</v>
       </c>
-      <c r="Q7" s="4" t="n">
+      <c r="Q7" s="8" t="n">
         <v>0.1419</v>
       </c>
-      <c r="R7" s="4" t="n">
+      <c r="R7" s="8" t="n">
         <v>0.1576</v>
       </c>
-      <c r="S7" s="4" t="n">
+      <c r="S7" s="8" t="n">
         <v>0.1465</v>
       </c>
-      <c r="T7" s="4" t="n">
+      <c r="T7" s="8" t="n">
         <v>0.1765</v>
       </c>
-      <c r="U7" s="4" t="n">
+      <c r="U7" s="8" t="n">
         <v>0.1697</v>
       </c>
-      <c r="V7" s="4" t="n">
+      <c r="V7" s="8" t="n">
         <v>0.1915</v>
       </c>
-      <c r="W7" s="4" t="n">
+      <c r="W7" s="8" t="n">
         <v>0.1558</v>
       </c>
     </row>
@@ -1745,70 +1970,70 @@
           <t>锐进1号</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="8" t="n">
         <v>0.0076</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="8" t="n">
         <v>0.009000000000000001</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="8" t="n">
         <v>0.0115</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="8" t="n">
         <v>0.0116</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="8" t="n">
         <v>0.0137</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="8" t="n">
         <v>0.0153</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="8" t="n">
         <v>0.0121</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="8" t="n">
         <v>0.0108</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="J8" s="8" t="n">
         <v>0.0139</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="K8" s="8" t="n">
         <v>0.008</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="L8" s="8" t="n">
         <v>0.0103</v>
       </c>
-      <c r="M8" s="4" t="n">
+      <c r="M8" s="8" t="n">
         <v>0.012</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="N8" s="8" t="n">
         <v>0.0142</v>
       </c>
-      <c r="O8" s="4" t="n">
+      <c r="O8" s="8" t="n">
         <v>0.0223</v>
       </c>
-      <c r="P8" s="4" t="n">
+      <c r="P8" s="8" t="n">
         <v>0.0243</v>
       </c>
-      <c r="Q8" s="4" t="n">
+      <c r="Q8" s="8" t="n">
         <v>0.0276</v>
       </c>
-      <c r="R8" s="4" t="n">
+      <c r="R8" s="8" t="n">
         <v>0.0267</v>
       </c>
-      <c r="S8" s="4" t="n">
+      <c r="S8" s="8" t="n">
         <v>0.0218</v>
       </c>
-      <c r="T8" s="4" t="n">
+      <c r="T8" s="8" t="n">
         <v>0.0323</v>
       </c>
-      <c r="U8" s="4" t="n">
+      <c r="U8" s="8" t="n">
         <v>0.0334</v>
       </c>
-      <c r="V8" s="4" t="n">
+      <c r="V8" s="8" t="n">
         <v>0.0421</v>
       </c>
-      <c r="W8" s="4" t="n">
+      <c r="W8" s="8" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -1974,70 +2199,70 @@
           <t>瑞享1号</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="G2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="M2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="N2" s="9" t="n">
         <v>4e-05</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="O2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="P2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="Q2" s="5" t="n">
+      <c r="Q2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="R2" s="5" t="n">
+      <c r="R2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="S2" s="5" t="n">
+      <c r="S2" s="9" t="n">
         <v>4e-05</v>
       </c>
-      <c r="T2" s="5" t="n">
+      <c r="T2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="U2" s="5" t="n">
+      <c r="U2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="V2" s="5" t="n">
+      <c r="V2" s="9" t="n">
         <v>5e-05</v>
       </c>
-      <c r="W2" s="5" t="n">
+      <c r="W2" s="9" t="n">
         <v>5e-05</v>
       </c>
     </row>
@@ -2047,70 +2272,70 @@
           <t>瑞享3号</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="9" t="n">
         <v>0.0307</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="9" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="9" t="n">
         <v>-0.0128</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="9" t="n">
         <v>-0.0118</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="9" t="n">
         <v>0.0048</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="9" t="n">
         <v>-0.0034</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="9" t="n">
         <v>0.0541</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="I3" s="9" t="n">
         <v>0.0495</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="9" t="n">
         <v>0.0147</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="K3" s="9" t="n">
         <v>-0.0392</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="9" t="n">
         <v>-0.0273</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="M3" s="9" t="n">
         <v>-0.0113</v>
       </c>
-      <c r="N3" s="5" t="n">
+      <c r="N3" s="9" t="n">
         <v>0.0004</v>
       </c>
-      <c r="O3" s="5" t="n">
+      <c r="O3" s="9" t="n">
         <v>-0.0244</v>
       </c>
-      <c r="P3" s="5" t="n">
+      <c r="P3" s="9" t="n">
         <v>0.0349</v>
       </c>
-      <c r="Q3" s="5" t="n">
+      <c r="Q3" s="9" t="n">
         <v>0.0129</v>
       </c>
-      <c r="R3" s="5" t="n">
+      <c r="R3" s="9" t="n">
         <v>0.0226</v>
       </c>
-      <c r="S3" s="5" t="n">
+      <c r="S3" s="9" t="n">
         <v>0.0063</v>
       </c>
-      <c r="T3" s="5" t="n">
+      <c r="T3" s="9" t="n">
         <v>-0.0185</v>
       </c>
-      <c r="U3" s="5" t="n">
+      <c r="U3" s="9" t="n">
         <v>-0.0038</v>
       </c>
-      <c r="V3" s="5" t="n">
+      <c r="V3" s="9" t="n">
         <v>0.0008</v>
       </c>
-      <c r="W3" s="5" t="n">
+      <c r="W3" s="9" t="n">
         <v>-0.0375</v>
       </c>
     </row>
@@ -2120,70 +2345,70 @@
           <t>配置1号</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="9" t="n">
         <v>0.0052</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="9" t="n">
         <v>0.0014</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="9" t="n">
         <v>0.0039</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="9" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="9" t="n">
         <v>0.004099999999999999</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="9" t="n">
         <v>-0.0028</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="9" t="n">
         <v>-0.0014</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="9" t="n">
         <v>0.0048</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="9" t="n">
         <v>-0.006500000000000001</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="9" t="n">
         <v>0.0019</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="M4" s="9" t="n">
         <v>0.0018</v>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="N4" s="9" t="n">
         <v>0.001</v>
       </c>
-      <c r="O4" s="5" t="n">
+      <c r="O4" s="9" t="n">
         <v>0.0107</v>
       </c>
-      <c r="P4" s="5" t="n">
+      <c r="P4" s="9" t="n">
         <v>0.0016</v>
       </c>
-      <c r="Q4" s="5" t="n">
+      <c r="Q4" s="9" t="n">
         <v>0.0064</v>
       </c>
-      <c r="R4" s="5" t="n">
+      <c r="R4" s="9" t="n">
         <v>0.0003</v>
       </c>
-      <c r="S4" s="5" t="n">
+      <c r="S4" s="9" t="n">
         <v>-0.0049</v>
       </c>
-      <c r="T4" s="5" t="n">
+      <c r="T4" s="9" t="n">
         <v>0.012</v>
       </c>
-      <c r="U4" s="5" t="n">
+      <c r="U4" s="9" t="n">
         <v>0.0004</v>
       </c>
-      <c r="V4" s="5" t="n">
+      <c r="V4" s="9" t="n">
         <v>0.009899999999999999</v>
       </c>
-      <c r="W4" s="5" t="n">
+      <c r="W4" s="9" t="n">
         <v>-0.0131</v>
       </c>
     </row>
@@ -2193,70 +2418,70 @@
           <t>瑞臻1号</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="9" t="n">
         <v>0.0193</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="9" t="n">
         <v>0.0063</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="9" t="n">
         <v>-0.0138</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="9" t="n">
         <v>-0.0275</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="9" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="9" t="n">
         <v>-0.008199999999999999</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="9" t="n">
         <v>0.0336</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I5" s="9" t="n">
         <v>0.05400000000000001</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="9" t="n">
         <v>-0.0075</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="9" t="n">
         <v>-0.0199</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="9" t="n">
         <v>-0.0104</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="9" t="n">
         <v>-0.0125</v>
       </c>
-      <c r="N5" s="5" t="n">
+      <c r="N5" s="9" t="n">
         <v>-0.0066</v>
       </c>
-      <c r="O5" s="5" t="n">
+      <c r="O5" s="9" t="n">
         <v>-0.0068</v>
       </c>
-      <c r="P5" s="5" t="n">
+      <c r="P5" s="9" t="n">
         <v>0.005500000000000001</v>
       </c>
-      <c r="Q5" s="5" t="n">
+      <c r="Q5" s="9" t="n">
         <v>0.0009</v>
       </c>
-      <c r="R5" s="5" t="n">
+      <c r="R5" s="9" t="n">
         <v>-0.005600000000000001</v>
       </c>
-      <c r="S5" s="5" t="n">
+      <c r="S5" s="9" t="n">
         <v>0.0222</v>
       </c>
-      <c r="T5" s="5" t="n">
+      <c r="T5" s="9" t="n">
         <v>0.0025</v>
       </c>
-      <c r="U5" s="5" t="n">
+      <c r="U5" s="9" t="n">
         <v>-0.0226</v>
       </c>
-      <c r="V5" s="5" t="n">
+      <c r="V5" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="W5" s="5" t="n">
+      <c r="W5" s="9" t="n">
         <v>-0.03700000000000001</v>
       </c>
     </row>
@@ -2266,70 +2491,70 @@
           <t>鑫盛1号</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.0068</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="9" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="9" t="n">
         <v>0.0051</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="9" t="n">
         <v>0.004699999999999999</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="9" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="9" t="n">
         <v>-0.002</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="9" t="n">
         <v>-0.0011</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="9" t="n">
         <v>0.0052</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="9" t="n">
         <v>-0.006500000000000001</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L6" s="9" t="n">
         <v>0.0019</v>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="M6" s="9" t="n">
         <v>0.0017</v>
       </c>
-      <c r="N6" s="5" t="n">
+      <c r="N6" s="9" t="n">
         <v>0.0016</v>
       </c>
-      <c r="O6" s="5" t="n">
+      <c r="O6" s="9" t="n">
         <v>0.0109</v>
       </c>
-      <c r="P6" s="5" t="n">
+      <c r="P6" s="9" t="n">
         <v>0.0019</v>
       </c>
-      <c r="Q6" s="5" t="n">
+      <c r="Q6" s="9" t="n">
         <v>0.008</v>
       </c>
-      <c r="R6" s="5" t="n">
+      <c r="R6" s="9" t="n">
         <v>0.0008</v>
       </c>
-      <c r="S6" s="5" t="n">
+      <c r="S6" s="9" t="n">
         <v>-0.0052</v>
       </c>
-      <c r="T6" s="5" t="n">
+      <c r="T6" s="9" t="n">
         <v>0.012</v>
       </c>
-      <c r="U6" s="5" t="n">
+      <c r="U6" s="9" t="n">
         <v>0.0011</v>
       </c>
-      <c r="V6" s="5" t="n">
+      <c r="V6" s="9" t="n">
         <v>0.0102</v>
       </c>
-      <c r="W6" s="5" t="n">
+      <c r="W6" s="9" t="n">
         <v>-0.0145</v>
       </c>
     </row>
@@ -2339,70 +2564,70 @@
           <t>领航1号</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="9" t="n">
         <v>0.0185</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="9" t="n">
         <v>0.0025</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="9" t="n">
         <v>0.0165</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="9" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="9" t="n">
         <v>0.0233</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="9" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="9" t="n">
         <v>0.004</v>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="I7" s="9" t="n">
         <v>0.0005</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J7" s="9" t="n">
         <v>0.014</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="9" t="n">
         <v>-0.0197</v>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="L7" s="9" t="n">
         <v>0.0027</v>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="M7" s="9" t="n">
         <v>0.0072</v>
       </c>
-      <c r="N7" s="5" t="n">
+      <c r="N7" s="9" t="n">
         <v>-0.0071</v>
       </c>
-      <c r="O7" s="5" t="n">
+      <c r="O7" s="9" t="n">
         <v>0.0306</v>
       </c>
-      <c r="P7" s="5" t="n">
+      <c r="P7" s="9" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="Q7" s="5" t="n">
+      <c r="Q7" s="9" t="n">
         <v>0.04099999999999999</v>
       </c>
-      <c r="R7" s="5" t="n">
+      <c r="R7" s="9" t="n">
         <v>0.0137</v>
       </c>
-      <c r="S7" s="5" t="n">
+      <c r="S7" s="9" t="n">
         <v>-0.009599999999999999</v>
       </c>
-      <c r="T7" s="5" t="n">
+      <c r="T7" s="9" t="n">
         <v>0.0263</v>
       </c>
-      <c r="U7" s="5" t="n">
+      <c r="U7" s="9" t="n">
         <v>-0.0058</v>
       </c>
-      <c r="V7" s="5" t="n">
+      <c r="V7" s="9" t="n">
         <v>0.0186</v>
       </c>
-      <c r="W7" s="5" t="n">
+      <c r="W7" s="9" t="n">
         <v>-0.03</v>
       </c>
     </row>
@@ -2412,289 +2637,289 @@
           <t>锐进1号</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.0039</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="9" t="n">
         <v>0.0014</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="9" t="n">
         <v>0.0025</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="9" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="9" t="n">
         <v>0.0022</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="9" t="n">
         <v>0.0015</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="9" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="9" t="n">
         <v>-0.0013</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="9" t="n">
         <v>0.0031</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="9" t="n">
         <v>-0.005699999999999999</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="L8" s="9" t="n">
         <v>0.0022</v>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="M8" s="9" t="n">
         <v>0.0018</v>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="N8" s="9" t="n">
         <v>0.0021</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="O8" s="9" t="n">
         <v>0.008</v>
       </c>
-      <c r="P8" s="5" t="n">
+      <c r="P8" s="9" t="n">
         <v>0.002</v>
       </c>
-      <c r="Q8" s="5" t="n">
+      <c r="Q8" s="9" t="n">
         <v>0.0034</v>
       </c>
-      <c r="R8" s="5" t="n">
+      <c r="R8" s="9" t="n">
         <v>-0.0009</v>
       </c>
-      <c r="S8" s="5" t="n">
+      <c r="S8" s="9" t="n">
         <v>-0.0048</v>
       </c>
-      <c r="T8" s="5" t="n">
+      <c r="T8" s="9" t="n">
         <v>0.0103</v>
       </c>
-      <c r="U8" s="5" t="n">
+      <c r="U8" s="9" t="n">
         <v>0.0012</v>
       </c>
-      <c r="V8" s="5" t="n">
+      <c r="V8" s="9" t="n">
         <v>0.0083</v>
       </c>
-      <c r="W8" s="5" t="n">
+      <c r="W8" s="9" t="n">
         <v>-0.0116</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>沪深300 (单日)</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="10" t="n">
         <v>0.01540480813500227</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="10" t="n">
         <v>0.002068147209394571</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="10" t="n">
         <v>0.0118655328430096</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="10" t="n">
         <v>-0.003411259779961792</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="10" t="n">
         <v>0.01096234767930233</v>
       </c>
-      <c r="G9" s="7" t="n">
+      <c r="G9" s="10" t="n">
         <v>-0.001675481801036615</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="10" t="n">
         <v>0.006084224584342067</v>
       </c>
-      <c r="I9" s="7" t="n">
+      <c r="I9" s="10" t="n">
         <v>0.002218650321299876</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="J9" s="10" t="n">
         <v>0.006633812898791696</v>
       </c>
-      <c r="K9" s="7" t="n">
+      <c r="K9" s="10" t="n">
         <v>-0.002770986162049777</v>
       </c>
-      <c r="L9" s="7" t="n">
+      <c r="L9" s="10" t="n">
         <v>-0.003543113317804182</v>
       </c>
-      <c r="M9" s="7" t="n">
+      <c r="M9" s="10" t="n">
         <v>0.0003308823591079226</v>
       </c>
-      <c r="N9" s="7" t="n">
+      <c r="N9" s="10" t="n">
         <v>-0.00267003600480225</v>
       </c>
-      <c r="O9" s="7" t="n">
+      <c r="O9" s="10" t="n">
         <v>0.01095759090664442</v>
       </c>
-      <c r="P9" s="7" t="n">
+      <c r="P9" s="10" t="n">
         <v>-0.0006319502785122833</v>
       </c>
-      <c r="Q9" s="7" t="n">
+      <c r="Q9" s="10" t="n">
         <v>0.01451671412948499</v>
       </c>
-      <c r="R9" s="7" t="n">
+      <c r="R9" s="10" t="n">
         <v>0.004801343554394154</v>
       </c>
-      <c r="S9" s="7" t="n">
+      <c r="S9" s="10" t="n">
         <v>-0.005835637753443541</v>
       </c>
-      <c r="T9" s="7" t="n">
+      <c r="T9" s="10" t="n">
         <v>0.01640513964927362</v>
       </c>
-      <c r="U9" s="7" t="n">
+      <c r="U9" s="10" t="n">
         <v>-0.0007653927837601216</v>
       </c>
-      <c r="V9" s="7" t="n">
+      <c r="V9" s="10" t="n">
         <v>0.01016465791095528</v>
       </c>
-      <c r="W9" s="7" t="n">
+      <c r="W9" s="10" t="n">
         <v>-0.0167544767897721</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>中证500 (单日)</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="10" t="n">
         <v>0.008954929403036351</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="10" t="n">
         <v>-0.000209251312206216</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="10" t="n">
         <v>0.0151702179437797</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="10" t="n">
         <v>-0.005500528171319097</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="10" t="n">
         <v>0.01690737109152349</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G10" s="10" t="n">
         <v>0.004170178500055284</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="10" t="n">
         <v>0.009231398835130933</v>
       </c>
-      <c r="I10" s="7" t="n">
+      <c r="I10" s="10" t="n">
         <v>-0.002375844002544493</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="10" t="n">
         <v>0.01279927687499061</v>
       </c>
-      <c r="K10" s="7" t="n">
+      <c r="K10" s="10" t="n">
         <v>-0.00966715045119367</v>
       </c>
-      <c r="L10" s="7" t="n">
+      <c r="L10" s="10" t="n">
         <v>-0.005705837117747784</v>
       </c>
-      <c r="M10" s="7" t="n">
+      <c r="M10" s="10" t="n">
         <v>0.006204348928189013</v>
       </c>
-      <c r="N10" s="7" t="n">
+      <c r="N10" s="10" t="n">
         <v>-0.01145760250156867</v>
       </c>
-      <c r="O10" s="7" t="n">
+      <c r="O10" s="10" t="n">
         <v>0.01687724908115738</v>
       </c>
-      <c r="P10" s="7" t="n">
+      <c r="P10" s="10" t="n">
         <v>0.0008494415955978729</v>
       </c>
-      <c r="Q10" s="7" t="n">
+      <c r="Q10" s="10" t="n">
         <v>0.02861627261610781</v>
       </c>
-      <c r="R10" s="7" t="n">
+      <c r="R10" s="10" t="n">
         <v>0.01261684325228851</v>
       </c>
-      <c r="S10" s="7" t="n">
+      <c r="S10" s="10" t="n">
         <v>-0.0003021801504460005</v>
       </c>
-      <c r="T10" s="7" t="n">
+      <c r="T10" s="10" t="n">
         <v>0.01674347119171547</v>
       </c>
-      <c r="U10" s="7" t="n">
+      <c r="U10" s="10" t="n">
         <v>-0.006081897304349864</v>
       </c>
-      <c r="V10" s="7" t="n">
+      <c r="V10" s="10" t="n">
         <v>0.01505351862264265</v>
       </c>
-      <c r="W10" s="7" t="n">
+      <c r="W10" s="10" t="n">
         <v>-0.02781733030478321</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>领航1号 - 中证500 超额</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="11" t="n">
         <v>0.00954507059696365</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="11" t="n">
         <v>0.002709251312206216</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="11" t="n">
         <v>0.001329782056220299</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="11" t="n">
         <v>0.006200528171319097</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="11" t="n">
         <v>0.006392628908476512</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="11" t="n">
         <v>-0.004870178500055284</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H11" s="11" t="n">
         <v>-0.005231398835130932</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I11" s="11" t="n">
         <v>0.002875844002544493</v>
       </c>
-      <c r="J11" s="9" t="n">
+      <c r="J11" s="11" t="n">
         <v>0.001200723125009384</v>
       </c>
-      <c r="K11" s="9" t="n">
+      <c r="K11" s="11" t="n">
         <v>-0.01003284954880633</v>
       </c>
-      <c r="L11" s="9" t="n">
+      <c r="L11" s="11" t="n">
         <v>0.008405837117747785</v>
       </c>
-      <c r="M11" s="9" t="n">
+      <c r="M11" s="11" t="n">
         <v>0.0009956510718109868</v>
       </c>
-      <c r="N11" s="9" t="n">
+      <c r="N11" s="11" t="n">
         <v>0.004357602501568667</v>
       </c>
-      <c r="O11" s="9" t="n">
+      <c r="O11" s="11" t="n">
         <v>0.01372275091884262</v>
       </c>
-      <c r="P11" s="9" t="n">
+      <c r="P11" s="11" t="n">
         <v>-0.0001494415955978729</v>
       </c>
-      <c r="Q11" s="9" t="n">
+      <c r="Q11" s="11" t="n">
         <v>0.01238372738389219</v>
       </c>
-      <c r="R11" s="9" t="n">
+      <c r="R11" s="11" t="n">
         <v>0.001083156747711493</v>
       </c>
-      <c r="S11" s="9" t="n">
+      <c r="S11" s="11" t="n">
         <v>-0.009297819849553999</v>
       </c>
-      <c r="T11" s="9" t="n">
+      <c r="T11" s="11" t="n">
         <v>0.009556528808284533</v>
       </c>
-      <c r="U11" s="9" t="n">
+      <c r="U11" s="11" t="n">
         <v>0.000281897304349864</v>
       </c>
-      <c r="V11" s="9" t="n">
+      <c r="V11" s="11" t="n">
         <v>0.003546481377357351</v>
       </c>
-      <c r="W11" s="9" t="n">
+      <c r="W11" s="11" t="n">
         <v>-0.002182669695216788</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Embed 领航1号 NAV vs cumulative-excess chart in NAV sheet
The 基金单位净值 sheet now carries a native Excel line chart: 领航1号
unit NAV on the primary (left) axis, 领航1号 - 中证500 累计超额 on a
secondary (right) axis. The excess row is now a live Excel formula
=(领航1号_d/领航1号_首日-1)-(中证500_d/中证500_首日-1) so the cells and
the chart recompute on edit, plus a visible formula caption.

https://claude.ai/code/session_014VmLcPuADdRYg34QDm2fTF
</commit_message>
<xml_diff>
--- a/output/20260410_20260514_table.xlsx
+++ b/output/20260410_20260514_table.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="009C0006"/>
+    </font>
+    <font>
+      <i val="1"/>
       <color rgb="009C0006"/>
     </font>
   </fonts>
@@ -95,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -118,6 +122,7 @@
     <xf numFmtId="10" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -204,6 +209,222 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>领航1号 单位净值 与 领航1号-中证500 累计超额</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'基金单位净值'!A7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="1F6FEB"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'基金单位净值'!$B$1:$W$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'基金单位净值'!$B$7:$W$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'基金单位净值'!A11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="26000">
+              <a:solidFill>
+                <a:srgbClr val="9C0006"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'基金单位净值'!$B$1:$W$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'基金单位净值'!$B$11:$W$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>日期</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>领航1号 单位净值</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>领航1号-中证500 累计超额 (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0.00%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6803999" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -495,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1303,75 +1524,108 @@
           <t>领航1号 - 中证500 累计超额</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>0.002564039381279914</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>0.003978628478572777</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>0.01024824559432114</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>0.01692648112621087</v>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>0.01195922630920832</v>
-      </c>
-      <c r="H11" s="7" t="n">
-        <v>0.006466989783670885</v>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>0.009429009822418566</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>0.01076567921138882</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>2.756948569748729e-05</v>
-      </c>
-      <c r="L11" s="7" t="n">
-        <v>0.008812069359058539</v>
-      </c>
-      <c r="M11" s="7" t="n">
-        <v>0.009847721329049319</v>
-      </c>
-      <c r="N11" s="7" t="n">
-        <v>0.01432248357702504</v>
-      </c>
-      <c r="O11" s="7" t="n">
-        <v>0.02893428464983949</v>
-      </c>
-      <c r="P11" s="7" t="n">
-        <v>0.02883000886178766</v>
-      </c>
-      <c r="Q11" s="7" t="n">
-        <v>0.04270665056181477</v>
-      </c>
-      <c r="R11" s="7" t="n">
-        <v>0.04451394570507161</v>
-      </c>
-      <c r="S11" s="7" t="n">
-        <v>0.03395281368752312</v>
-      </c>
-      <c r="T11" s="7" t="n">
-        <v>0.04512139022337847</v>
-      </c>
-      <c r="U11" s="7" t="n">
-        <v>0.04519562450781467</v>
-      </c>
-      <c r="V11" s="7" t="n">
-        <v>0.04998890867505268</v>
-      </c>
-      <c r="W11" s="7" t="n">
-        <v>0.0460908438797849</v>
+      <c r="B11" s="7">
+        <f>(B7/$B$7-1)-(B10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="C11" s="7">
+        <f>(C7/$B$7-1)-(C10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="D11" s="7">
+        <f>(D7/$B$7-1)-(D10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="E11" s="7">
+        <f>(E7/$B$7-1)-(E10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="F11" s="7">
+        <f>(F7/$B$7-1)-(F10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="G11" s="7">
+        <f>(G7/$B$7-1)-(G10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="H11" s="7">
+        <f>(H7/$B$7-1)-(H10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="I11" s="7">
+        <f>(I7/$B$7-1)-(I10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="J11" s="7">
+        <f>(J7/$B$7-1)-(J10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="K11" s="7">
+        <f>(K7/$B$7-1)-(K10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="L11" s="7">
+        <f>(L7/$B$7-1)-(L10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="M11" s="7">
+        <f>(M7/$B$7-1)-(M10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="N11" s="7">
+        <f>(N7/$B$7-1)-(N10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="O11" s="7">
+        <f>(O7/$B$7-1)-(O10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="P11" s="7">
+        <f>(P7/$B$7-1)-(P10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="7">
+        <f>(Q7/$B$7-1)-(Q10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="R11" s="7">
+        <f>(R7/$B$7-1)-(R10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="S11" s="7">
+        <f>(S7/$B$7-1)-(S10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="T11" s="7">
+        <f>(T7/$B$7-1)-(T10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="U11" s="7">
+        <f>(U7/$B$7-1)-(U10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="V11" s="7">
+        <f>(V7/$B$7-1)-(V10/$B$10-1)</f>
+        <v/>
+      </c>
+      <c r="W11" s="7">
+        <f>(W7/$B$7-1)-(W10/$B$10-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>累计超额 = (领航1号净值 ÷ 首日净值 − 1) − (中证500收盘 ÷ 首日收盘 − 1)；首日 = 0，单位：百分点</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:L13"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1532,70 +1786,70 @@
           <t>瑞享1号</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="9" t="n">
         <v>0.0062</v>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="9" t="n">
         <v>0.0064</v>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D2" s="9" t="n">
         <v>0.0064</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E2" s="9" t="n">
         <v>0.006500000000000001</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="9" t="n">
         <v>0.006500000000000001</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="9" t="n">
         <v>0.0066</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="9" t="n">
         <v>0.0067</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="9" t="n">
         <v>0.0067</v>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="J2" s="9" t="n">
         <v>0.0068</v>
       </c>
-      <c r="K2" s="8" t="n">
+      <c r="K2" s="9" t="n">
         <v>0.0068</v>
       </c>
-      <c r="L2" s="8" t="n">
+      <c r="L2" s="9" t="n">
         <v>0.0069</v>
       </c>
-      <c r="M2" s="8" t="n">
+      <c r="M2" s="9" t="n">
         <v>0.006999999999999999</v>
       </c>
-      <c r="N2" s="8" t="n">
+      <c r="N2" s="9" t="n">
         <v>0.0071</v>
       </c>
-      <c r="O2" s="8" t="n">
+      <c r="O2" s="9" t="n">
         <v>0.0071</v>
       </c>
-      <c r="P2" s="8" t="n">
+      <c r="P2" s="9" t="n">
         <v>0.0072</v>
       </c>
-      <c r="Q2" s="8" t="n">
+      <c r="Q2" s="9" t="n">
         <v>0.0075</v>
       </c>
-      <c r="R2" s="8" t="n">
+      <c r="R2" s="9" t="n">
         <v>0.0075</v>
       </c>
-      <c r="S2" s="8" t="n">
+      <c r="S2" s="9" t="n">
         <v>0.0076</v>
       </c>
-      <c r="T2" s="8" t="n">
+      <c r="T2" s="9" t="n">
         <v>0.0077</v>
       </c>
-      <c r="U2" s="8" t="n">
+      <c r="U2" s="9" t="n">
         <v>0.0077</v>
       </c>
-      <c r="V2" s="8" t="n">
+      <c r="V2" s="9" t="n">
         <v>0.007800000000000001</v>
       </c>
-      <c r="W2" s="8" t="n">
+      <c r="W2" s="9" t="n">
         <v>0.007800000000000001</v>
       </c>
     </row>
@@ -1605,70 +1859,70 @@
           <t>瑞享3号</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="9" t="n">
         <v>-0.163</v>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="9" t="n">
         <v>-0.1637</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="9" t="n">
         <v>-0.1743</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="9" t="n">
         <v>-0.1841</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="9" t="n">
         <v>-0.1802</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="9" t="n">
         <v>-0.183</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="9" t="n">
         <v>-0.1389</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="9" t="n">
         <v>-0.09619999999999999</v>
       </c>
-      <c r="J3" s="8" t="n">
+      <c r="J3" s="9" t="n">
         <v>-0.083</v>
       </c>
-      <c r="K3" s="8" t="n">
+      <c r="K3" s="9" t="n">
         <v>-0.1189</v>
       </c>
-      <c r="L3" s="8" t="n">
+      <c r="L3" s="9" t="n">
         <v>-0.1429</v>
       </c>
-      <c r="M3" s="8" t="n">
+      <c r="M3" s="9" t="n">
         <v>-0.1527</v>
       </c>
-      <c r="N3" s="8" t="n">
+      <c r="N3" s="9" t="n">
         <v>-0.1523</v>
       </c>
-      <c r="O3" s="8" t="n">
+      <c r="O3" s="9" t="n">
         <v>-0.173</v>
       </c>
-      <c r="P3" s="8" t="n">
+      <c r="P3" s="9" t="n">
         <v>-0.1441</v>
       </c>
-      <c r="Q3" s="8" t="n">
+      <c r="Q3" s="9" t="n">
         <v>-0.1333</v>
       </c>
-      <c r="R3" s="8" t="n">
+      <c r="R3" s="9" t="n">
         <v>-0.1136</v>
       </c>
-      <c r="S3" s="8" t="n">
+      <c r="S3" s="9" t="n">
         <v>-0.1081</v>
       </c>
-      <c r="T3" s="8" t="n">
+      <c r="T3" s="9" t="n">
         <v>-0.1246</v>
       </c>
-      <c r="U3" s="8" t="n">
+      <c r="U3" s="9" t="n">
         <v>-0.1279</v>
       </c>
-      <c r="V3" s="8" t="n">
+      <c r="V3" s="9" t="n">
         <v>-0.1272</v>
       </c>
-      <c r="W3" s="8" t="n">
+      <c r="W3" s="9" t="n">
         <v>-0.1599</v>
       </c>
     </row>
@@ -1678,70 +1932,70 @@
           <t>配置1号</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <v>0.0104</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="9" t="n">
         <v>0.0117</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="9" t="n">
         <v>0.0156</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="9" t="n">
         <v>0.0159</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="F4" s="9" t="n">
         <v>0.02</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="9" t="n">
         <v>0.0212</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="9" t="n">
         <v>0.0183</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="9" t="n">
         <v>0.0169</v>
       </c>
-      <c r="J4" s="8" t="n">
+      <c r="J4" s="9" t="n">
         <v>0.0218</v>
       </c>
-      <c r="K4" s="8" t="n">
+      <c r="K4" s="9" t="n">
         <v>0.0151</v>
       </c>
-      <c r="L4" s="8" t="n">
+      <c r="L4" s="9" t="n">
         <v>0.0171</v>
       </c>
-      <c r="M4" s="8" t="n">
+      <c r="M4" s="9" t="n">
         <v>0.0188</v>
       </c>
-      <c r="N4" s="8" t="n">
+      <c r="N4" s="9" t="n">
         <v>0.0198</v>
       </c>
-      <c r="O4" s="8" t="n">
+      <c r="O4" s="9" t="n">
         <v>0.0307</v>
       </c>
-      <c r="P4" s="8" t="n">
+      <c r="P4" s="9" t="n">
         <v>0.0323</v>
       </c>
-      <c r="Q4" s="8" t="n">
+      <c r="Q4" s="9" t="n">
         <v>0.0388</v>
       </c>
-      <c r="R4" s="8" t="n">
+      <c r="R4" s="9" t="n">
         <v>0.039</v>
       </c>
-      <c r="S4" s="8" t="n">
+      <c r="S4" s="9" t="n">
         <v>0.0339</v>
       </c>
-      <c r="T4" s="8" t="n">
+      <c r="T4" s="9" t="n">
         <v>0.0463</v>
       </c>
-      <c r="U4" s="8" t="n">
+      <c r="U4" s="9" t="n">
         <v>0.0467</v>
       </c>
-      <c r="V4" s="8" t="n">
+      <c r="V4" s="9" t="n">
         <v>0.057</v>
       </c>
-      <c r="W4" s="8" t="n">
+      <c r="W4" s="9" t="n">
         <v>0.0432</v>
       </c>
     </row>
@@ -1751,70 +2005,70 @@
           <t>瑞臻1号</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>-0.09570000000000001</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="9" t="n">
         <v>-0.0901</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="9" t="n">
         <v>-0.1026</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="9" t="n">
         <v>-0.1273</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="9" t="n">
         <v>-0.1301</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="9" t="n">
         <v>-0.1372</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="9" t="n">
         <v>-0.1083</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="9" t="n">
         <v>-0.0604</v>
       </c>
-      <c r="J5" s="8" t="n">
+      <c r="J5" s="9" t="n">
         <v>-0.0673</v>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="K5" s="9" t="n">
         <v>-0.0858</v>
       </c>
-      <c r="L5" s="8" t="n">
+      <c r="L5" s="9" t="n">
         <v>-0.0953</v>
       </c>
-      <c r="M5" s="8" t="n">
+      <c r="M5" s="9" t="n">
         <v>-0.1067</v>
       </c>
-      <c r="N5" s="8" t="n">
+      <c r="N5" s="9" t="n">
         <v>-0.1126</v>
       </c>
-      <c r="O5" s="8" t="n">
+      <c r="O5" s="9" t="n">
         <v>-0.1186</v>
       </c>
-      <c r="P5" s="8" t="n">
+      <c r="P5" s="9" t="n">
         <v>-0.1137</v>
       </c>
-      <c r="Q5" s="8" t="n">
+      <c r="Q5" s="9" t="n">
         <v>-0.1131</v>
       </c>
-      <c r="R5" s="8" t="n">
+      <c r="R5" s="9" t="n">
         <v>-0.1181</v>
       </c>
-      <c r="S5" s="8" t="n">
+      <c r="S5" s="9" t="n">
         <v>-0.09859999999999999</v>
       </c>
-      <c r="T5" s="8" t="n">
+      <c r="T5" s="9" t="n">
         <v>-0.0964</v>
       </c>
-      <c r="U5" s="8" t="n">
+      <c r="U5" s="9" t="n">
         <v>-0.1168</v>
       </c>
-      <c r="V5" s="8" t="n">
+      <c r="V5" s="9" t="n">
         <v>-0.1158</v>
       </c>
-      <c r="W5" s="8" t="n">
+      <c r="W5" s="9" t="n">
         <v>-0.1485</v>
       </c>
     </row>
@@ -1824,70 +2078,70 @@
           <t>鑫盛1号</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.1378</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <v>0.1385</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="9" t="n">
         <v>0.1443</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="9" t="n">
         <v>0.1455</v>
       </c>
-      <c r="F6" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <v>0.1509</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <v>0.1517</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="9" t="n">
         <v>0.1493</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="9" t="n">
         <v>0.148</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="9" t="n">
         <v>0.154</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K6" s="9" t="n">
         <v>0.1465</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="L6" s="9" t="n">
         <v>0.1486</v>
       </c>
-      <c r="M6" s="8" t="n">
+      <c r="M6" s="9" t="n">
         <v>0.1506</v>
       </c>
-      <c r="N6" s="8" t="n">
+      <c r="N6" s="9" t="n">
         <v>0.1524</v>
       </c>
-      <c r="O6" s="8" t="n">
+      <c r="O6" s="9" t="n">
         <v>0.1649</v>
       </c>
-      <c r="P6" s="8" t="n">
+      <c r="P6" s="9" t="n">
         <v>0.1671</v>
       </c>
-      <c r="Q6" s="8" t="n">
+      <c r="Q6" s="9" t="n">
         <v>0.1764</v>
       </c>
-      <c r="R6" s="8" t="n">
+      <c r="R6" s="9" t="n">
         <v>0.1774</v>
       </c>
-      <c r="S6" s="8" t="n">
+      <c r="S6" s="9" t="n">
         <v>0.1712</v>
       </c>
-      <c r="T6" s="8" t="n">
+      <c r="T6" s="9" t="n">
         <v>0.1853</v>
       </c>
-      <c r="U6" s="8" t="n">
+      <c r="U6" s="9" t="n">
         <v>0.1867</v>
       </c>
-      <c r="V6" s="8" t="n">
+      <c r="V6" s="9" t="n">
         <v>0.1987</v>
       </c>
-      <c r="W6" s="8" t="n">
+      <c r="W6" s="9" t="n">
         <v>0.1813</v>
       </c>
     </row>
@@ -1897,70 +2151,70 @@
           <t>领航1号</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>0.0191</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <v>0.0216</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>0.0385</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <v>0.0392</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <v>0.0633</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="9" t="n">
         <v>0.0626</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="9" t="n">
         <v>0.0668</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="9" t="n">
         <v>0.0673</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="9" t="n">
         <v>0.08220000000000001</v>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="K7" s="9" t="n">
         <v>0.0609</v>
       </c>
-      <c r="L7" s="8" t="n">
+      <c r="L7" s="9" t="n">
         <v>0.0638</v>
       </c>
-      <c r="M7" s="8" t="n">
+      <c r="M7" s="9" t="n">
         <v>0.07139999999999999</v>
       </c>
-      <c r="N7" s="8" t="n">
+      <c r="N7" s="9" t="n">
         <v>0.0638</v>
       </c>
-      <c r="O7" s="8" t="n">
+      <c r="O7" s="9" t="n">
         <v>0.0964</v>
       </c>
-      <c r="P7" s="8" t="n">
+      <c r="P7" s="9" t="n">
         <v>0.09710000000000001</v>
       </c>
-      <c r="Q7" s="8" t="n">
+      <c r="Q7" s="9" t="n">
         <v>0.1419</v>
       </c>
-      <c r="R7" s="8" t="n">
+      <c r="R7" s="9" t="n">
         <v>0.1576</v>
       </c>
-      <c r="S7" s="8" t="n">
+      <c r="S7" s="9" t="n">
         <v>0.1465</v>
       </c>
-      <c r="T7" s="8" t="n">
+      <c r="T7" s="9" t="n">
         <v>0.1765</v>
       </c>
-      <c r="U7" s="8" t="n">
+      <c r="U7" s="9" t="n">
         <v>0.1697</v>
       </c>
-      <c r="V7" s="8" t="n">
+      <c r="V7" s="9" t="n">
         <v>0.1915</v>
       </c>
-      <c r="W7" s="8" t="n">
+      <c r="W7" s="9" t="n">
         <v>0.1558</v>
       </c>
     </row>
@@ -1970,70 +2224,70 @@
           <t>锐进1号</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.0076</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <v>0.009000000000000001</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <v>0.0115</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <v>0.0116</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>0.0137</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <v>0.0153</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <v>0.0121</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="9" t="n">
         <v>0.0108</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="9" t="n">
         <v>0.0139</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="K8" s="9" t="n">
         <v>0.008</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="L8" s="9" t="n">
         <v>0.0103</v>
       </c>
-      <c r="M8" s="8" t="n">
+      <c r="M8" s="9" t="n">
         <v>0.012</v>
       </c>
-      <c r="N8" s="8" t="n">
+      <c r="N8" s="9" t="n">
         <v>0.0142</v>
       </c>
-      <c r="O8" s="8" t="n">
+      <c r="O8" s="9" t="n">
         <v>0.0223</v>
       </c>
-      <c r="P8" s="8" t="n">
+      <c r="P8" s="9" t="n">
         <v>0.0243</v>
       </c>
-      <c r="Q8" s="8" t="n">
+      <c r="Q8" s="9" t="n">
         <v>0.0276</v>
       </c>
-      <c r="R8" s="8" t="n">
+      <c r="R8" s="9" t="n">
         <v>0.0267</v>
       </c>
-      <c r="S8" s="8" t="n">
+      <c r="S8" s="9" t="n">
         <v>0.0218</v>
       </c>
-      <c r="T8" s="8" t="n">
+      <c r="T8" s="9" t="n">
         <v>0.0323</v>
       </c>
-      <c r="U8" s="8" t="n">
+      <c r="U8" s="9" t="n">
         <v>0.0334</v>
       </c>
-      <c r="V8" s="8" t="n">
+      <c r="V8" s="9" t="n">
         <v>0.0421</v>
       </c>
-      <c r="W8" s="8" t="n">
+      <c r="W8" s="9" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -2199,70 +2453,70 @@
           <t>瑞享1号</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="F2" s="9" t="n">
+      <c r="F2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="G2" s="9" t="n">
+      <c r="G2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="H2" s="9" t="n">
+      <c r="H2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="I2" s="9" t="n">
+      <c r="I2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="J2" s="9" t="n">
+      <c r="J2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="K2" s="9" t="n">
+      <c r="K2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="L2" s="9" t="n">
+      <c r="L2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="M2" s="9" t="n">
+      <c r="M2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="N2" s="9" t="n">
+      <c r="N2" s="10" t="n">
         <v>4e-05</v>
       </c>
-      <c r="O2" s="9" t="n">
+      <c r="O2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="P2" s="9" t="n">
+      <c r="P2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="Q2" s="9" t="n">
+      <c r="Q2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="R2" s="9" t="n">
+      <c r="R2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="S2" s="9" t="n">
+      <c r="S2" s="10" t="n">
         <v>4e-05</v>
       </c>
-      <c r="T2" s="9" t="n">
+      <c r="T2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="U2" s="9" t="n">
+      <c r="U2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="V2" s="9" t="n">
+      <c r="V2" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="W2" s="9" t="n">
+      <c r="W2" s="10" t="n">
         <v>5e-05</v>
       </c>
     </row>
@@ -2272,70 +2526,70 @@
           <t>瑞享3号</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="10" t="n">
         <v>0.0307</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="10" t="n">
         <v>-0.0128</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="10" t="n">
         <v>-0.0118</v>
       </c>
-      <c r="F3" s="9" t="n">
+      <c r="F3" s="10" t="n">
         <v>0.0048</v>
       </c>
-      <c r="G3" s="9" t="n">
+      <c r="G3" s="10" t="n">
         <v>-0.0034</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="10" t="n">
         <v>0.0541</v>
       </c>
-      <c r="I3" s="9" t="n">
+      <c r="I3" s="10" t="n">
         <v>0.0495</v>
       </c>
-      <c r="J3" s="9" t="n">
+      <c r="J3" s="10" t="n">
         <v>0.0147</v>
       </c>
-      <c r="K3" s="9" t="n">
+      <c r="K3" s="10" t="n">
         <v>-0.0392</v>
       </c>
-      <c r="L3" s="9" t="n">
+      <c r="L3" s="10" t="n">
         <v>-0.0273</v>
       </c>
-      <c r="M3" s="9" t="n">
+      <c r="M3" s="10" t="n">
         <v>-0.0113</v>
       </c>
-      <c r="N3" s="9" t="n">
+      <c r="N3" s="10" t="n">
         <v>0.0004</v>
       </c>
-      <c r="O3" s="9" t="n">
+      <c r="O3" s="10" t="n">
         <v>-0.0244</v>
       </c>
-      <c r="P3" s="9" t="n">
+      <c r="P3" s="10" t="n">
         <v>0.0349</v>
       </c>
-      <c r="Q3" s="9" t="n">
+      <c r="Q3" s="10" t="n">
         <v>0.0129</v>
       </c>
-      <c r="R3" s="9" t="n">
+      <c r="R3" s="10" t="n">
         <v>0.0226</v>
       </c>
-      <c r="S3" s="9" t="n">
+      <c r="S3" s="10" t="n">
         <v>0.0063</v>
       </c>
-      <c r="T3" s="9" t="n">
+      <c r="T3" s="10" t="n">
         <v>-0.0185</v>
       </c>
-      <c r="U3" s="9" t="n">
+      <c r="U3" s="10" t="n">
         <v>-0.0038</v>
       </c>
-      <c r="V3" s="9" t="n">
+      <c r="V3" s="10" t="n">
         <v>0.0008</v>
       </c>
-      <c r="W3" s="9" t="n">
+      <c r="W3" s="10" t="n">
         <v>-0.0375</v>
       </c>
     </row>
@@ -2345,70 +2599,70 @@
           <t>配置1号</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="10" t="n">
         <v>0.0052</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="10" t="n">
         <v>0.0014</v>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="10" t="n">
         <v>0.0039</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="10" t="n">
         <v>0.0003</v>
       </c>
-      <c r="F4" s="9" t="n">
+      <c r="F4" s="10" t="n">
         <v>0.004099999999999999</v>
       </c>
-      <c r="G4" s="9" t="n">
+      <c r="G4" s="10" t="n">
         <v>0.0011</v>
       </c>
-      <c r="H4" s="9" t="n">
+      <c r="H4" s="10" t="n">
         <v>-0.0028</v>
       </c>
-      <c r="I4" s="9" t="n">
+      <c r="I4" s="10" t="n">
         <v>-0.0014</v>
       </c>
-      <c r="J4" s="9" t="n">
+      <c r="J4" s="10" t="n">
         <v>0.0048</v>
       </c>
-      <c r="K4" s="9" t="n">
+      <c r="K4" s="10" t="n">
         <v>-0.006500000000000001</v>
       </c>
-      <c r="L4" s="9" t="n">
+      <c r="L4" s="10" t="n">
         <v>0.0019</v>
       </c>
-      <c r="M4" s="9" t="n">
+      <c r="M4" s="10" t="n">
         <v>0.0018</v>
       </c>
-      <c r="N4" s="9" t="n">
+      <c r="N4" s="10" t="n">
         <v>0.001</v>
       </c>
-      <c r="O4" s="9" t="n">
+      <c r="O4" s="10" t="n">
         <v>0.0107</v>
       </c>
-      <c r="P4" s="9" t="n">
+      <c r="P4" s="10" t="n">
         <v>0.0016</v>
       </c>
-      <c r="Q4" s="9" t="n">
+      <c r="Q4" s="10" t="n">
         <v>0.0064</v>
       </c>
-      <c r="R4" s="9" t="n">
+      <c r="R4" s="10" t="n">
         <v>0.0003</v>
       </c>
-      <c r="S4" s="9" t="n">
+      <c r="S4" s="10" t="n">
         <v>-0.0049</v>
       </c>
-      <c r="T4" s="9" t="n">
+      <c r="T4" s="10" t="n">
         <v>0.012</v>
       </c>
-      <c r="U4" s="9" t="n">
+      <c r="U4" s="10" t="n">
         <v>0.0004</v>
       </c>
-      <c r="V4" s="9" t="n">
+      <c r="V4" s="10" t="n">
         <v>0.009899999999999999</v>
       </c>
-      <c r="W4" s="9" t="n">
+      <c r="W4" s="10" t="n">
         <v>-0.0131</v>
       </c>
     </row>
@@ -2418,70 +2672,70 @@
           <t>瑞臻1号</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="10" t="n">
         <v>0.0193</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10" t="n">
         <v>0.0063</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>-0.0138</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="10" t="n">
         <v>-0.0275</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="10" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="10" t="n">
         <v>-0.008199999999999999</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="10" t="n">
         <v>0.0336</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="10" t="n">
         <v>0.05400000000000001</v>
       </c>
-      <c r="J5" s="9" t="n">
+      <c r="J5" s="10" t="n">
         <v>-0.0075</v>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="K5" s="10" t="n">
         <v>-0.0199</v>
       </c>
-      <c r="L5" s="9" t="n">
+      <c r="L5" s="10" t="n">
         <v>-0.0104</v>
       </c>
-      <c r="M5" s="9" t="n">
+      <c r="M5" s="10" t="n">
         <v>-0.0125</v>
       </c>
-      <c r="N5" s="9" t="n">
+      <c r="N5" s="10" t="n">
         <v>-0.0066</v>
       </c>
-      <c r="O5" s="9" t="n">
+      <c r="O5" s="10" t="n">
         <v>-0.0068</v>
       </c>
-      <c r="P5" s="9" t="n">
+      <c r="P5" s="10" t="n">
         <v>0.005500000000000001</v>
       </c>
-      <c r="Q5" s="9" t="n">
+      <c r="Q5" s="10" t="n">
         <v>0.0009</v>
       </c>
-      <c r="R5" s="9" t="n">
+      <c r="R5" s="10" t="n">
         <v>-0.005600000000000001</v>
       </c>
-      <c r="S5" s="9" t="n">
+      <c r="S5" s="10" t="n">
         <v>0.0222</v>
       </c>
-      <c r="T5" s="9" t="n">
+      <c r="T5" s="10" t="n">
         <v>0.0025</v>
       </c>
-      <c r="U5" s="9" t="n">
+      <c r="U5" s="10" t="n">
         <v>-0.0226</v>
       </c>
-      <c r="V5" s="9" t="n">
+      <c r="V5" s="10" t="n">
         <v>0.0012</v>
       </c>
-      <c r="W5" s="9" t="n">
+      <c r="W5" s="10" t="n">
         <v>-0.03700000000000001</v>
       </c>
     </row>
@@ -2491,70 +2745,70 @@
           <t>鑫盛1号</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <v>0.0068</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="10" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="10" t="n">
         <v>0.0051</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="10" t="n">
         <v>0.0011</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="F6" s="10" t="n">
         <v>0.004699999999999999</v>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G6" s="10" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="10" t="n">
         <v>-0.002</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="10" t="n">
         <v>-0.0011</v>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="J6" s="10" t="n">
         <v>0.0052</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="10" t="n">
         <v>-0.006500000000000001</v>
       </c>
-      <c r="L6" s="9" t="n">
+      <c r="L6" s="10" t="n">
         <v>0.0019</v>
       </c>
-      <c r="M6" s="9" t="n">
+      <c r="M6" s="10" t="n">
         <v>0.0017</v>
       </c>
-      <c r="N6" s="9" t="n">
+      <c r="N6" s="10" t="n">
         <v>0.0016</v>
       </c>
-      <c r="O6" s="9" t="n">
+      <c r="O6" s="10" t="n">
         <v>0.0109</v>
       </c>
-      <c r="P6" s="9" t="n">
+      <c r="P6" s="10" t="n">
         <v>0.0019</v>
       </c>
-      <c r="Q6" s="9" t="n">
+      <c r="Q6" s="10" t="n">
         <v>0.008</v>
       </c>
-      <c r="R6" s="9" t="n">
+      <c r="R6" s="10" t="n">
         <v>0.0008</v>
       </c>
-      <c r="S6" s="9" t="n">
+      <c r="S6" s="10" t="n">
         <v>-0.0052</v>
       </c>
-      <c r="T6" s="9" t="n">
+      <c r="T6" s="10" t="n">
         <v>0.012</v>
       </c>
-      <c r="U6" s="9" t="n">
+      <c r="U6" s="10" t="n">
         <v>0.0011</v>
       </c>
-      <c r="V6" s="9" t="n">
+      <c r="V6" s="10" t="n">
         <v>0.0102</v>
       </c>
-      <c r="W6" s="9" t="n">
+      <c r="W6" s="10" t="n">
         <v>-0.0145</v>
       </c>
     </row>
@@ -2564,70 +2818,70 @@
           <t>领航1号</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <v>0.0185</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="10" t="n">
         <v>0.0025</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <v>0.0165</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="10" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="10" t="n">
         <v>0.0233</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="10" t="n">
         <v>-0.0007000000000000001</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="10" t="n">
         <v>0.004</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I7" s="10" t="n">
         <v>0.0005</v>
       </c>
-      <c r="J7" s="9" t="n">
+      <c r="J7" s="10" t="n">
         <v>0.014</v>
       </c>
-      <c r="K7" s="9" t="n">
+      <c r="K7" s="10" t="n">
         <v>-0.0197</v>
       </c>
-      <c r="L7" s="9" t="n">
+      <c r="L7" s="10" t="n">
         <v>0.0027</v>
       </c>
-      <c r="M7" s="9" t="n">
+      <c r="M7" s="10" t="n">
         <v>0.0072</v>
       </c>
-      <c r="N7" s="9" t="n">
+      <c r="N7" s="10" t="n">
         <v>-0.0071</v>
       </c>
-      <c r="O7" s="9" t="n">
+      <c r="O7" s="10" t="n">
         <v>0.0306</v>
       </c>
-      <c r="P7" s="9" t="n">
+      <c r="P7" s="10" t="n">
         <v>0.0007000000000000001</v>
       </c>
-      <c r="Q7" s="9" t="n">
+      <c r="Q7" s="10" t="n">
         <v>0.04099999999999999</v>
       </c>
-      <c r="R7" s="9" t="n">
+      <c r="R7" s="10" t="n">
         <v>0.0137</v>
       </c>
-      <c r="S7" s="9" t="n">
+      <c r="S7" s="10" t="n">
         <v>-0.009599999999999999</v>
       </c>
-      <c r="T7" s="9" t="n">
+      <c r="T7" s="10" t="n">
         <v>0.0263</v>
       </c>
-      <c r="U7" s="9" t="n">
+      <c r="U7" s="10" t="n">
         <v>-0.0058</v>
       </c>
-      <c r="V7" s="9" t="n">
+      <c r="V7" s="10" t="n">
         <v>0.0186</v>
       </c>
-      <c r="W7" s="9" t="n">
+      <c r="W7" s="10" t="n">
         <v>-0.03</v>
       </c>
     </row>
@@ -2637,70 +2891,70 @@
           <t>锐进1号</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <v>0.0039</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10" t="n">
         <v>0.0014</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10" t="n">
         <v>0.0025</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="10" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="10" t="n">
         <v>0.0022</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G8" s="10" t="n">
         <v>0.0015</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="10" t="n">
         <v>-0.0032</v>
       </c>
-      <c r="I8" s="9" t="n">
+      <c r="I8" s="10" t="n">
         <v>-0.0013</v>
       </c>
-      <c r="J8" s="9" t="n">
+      <c r="J8" s="10" t="n">
         <v>0.0031</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="K8" s="10" t="n">
         <v>-0.005699999999999999</v>
       </c>
-      <c r="L8" s="9" t="n">
+      <c r="L8" s="10" t="n">
         <v>0.0022</v>
       </c>
-      <c r="M8" s="9" t="n">
+      <c r="M8" s="10" t="n">
         <v>0.0018</v>
       </c>
-      <c r="N8" s="9" t="n">
+      <c r="N8" s="10" t="n">
         <v>0.0021</v>
       </c>
-      <c r="O8" s="9" t="n">
+      <c r="O8" s="10" t="n">
         <v>0.008</v>
       </c>
-      <c r="P8" s="9" t="n">
+      <c r="P8" s="10" t="n">
         <v>0.002</v>
       </c>
-      <c r="Q8" s="9" t="n">
+      <c r="Q8" s="10" t="n">
         <v>0.0034</v>
       </c>
-      <c r="R8" s="9" t="n">
+      <c r="R8" s="10" t="n">
         <v>-0.0009</v>
       </c>
-      <c r="S8" s="9" t="n">
+      <c r="S8" s="10" t="n">
         <v>-0.0048</v>
       </c>
-      <c r="T8" s="9" t="n">
+      <c r="T8" s="10" t="n">
         <v>0.0103</v>
       </c>
-      <c r="U8" s="9" t="n">
+      <c r="U8" s="10" t="n">
         <v>0.0012</v>
       </c>
-      <c r="V8" s="9" t="n">
+      <c r="V8" s="10" t="n">
         <v>0.0083</v>
       </c>
-      <c r="W8" s="9" t="n">
+      <c r="W8" s="10" t="n">
         <v>-0.0116</v>
       </c>
     </row>
@@ -2710,70 +2964,70 @@
           <t>沪深300 (单日)</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>0.01540480813500227</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>0.002068147209394571</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <v>0.0118655328430096</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <v>-0.003411259779961792</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="11" t="n">
         <v>0.01096234767930233</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="11" t="n">
         <v>-0.001675481801036615</v>
       </c>
-      <c r="H9" s="10" t="n">
+      <c r="H9" s="11" t="n">
         <v>0.006084224584342067</v>
       </c>
-      <c r="I9" s="10" t="n">
+      <c r="I9" s="11" t="n">
         <v>0.002218650321299876</v>
       </c>
-      <c r="J9" s="10" t="n">
+      <c r="J9" s="11" t="n">
         <v>0.006633812898791696</v>
       </c>
-      <c r="K9" s="10" t="n">
+      <c r="K9" s="11" t="n">
         <v>-0.002770986162049777</v>
       </c>
-      <c r="L9" s="10" t="n">
+      <c r="L9" s="11" t="n">
         <v>-0.003543113317804182</v>
       </c>
-      <c r="M9" s="10" t="n">
+      <c r="M9" s="11" t="n">
         <v>0.0003308823591079226</v>
       </c>
-      <c r="N9" s="10" t="n">
+      <c r="N9" s="11" t="n">
         <v>-0.00267003600480225</v>
       </c>
-      <c r="O9" s="10" t="n">
+      <c r="O9" s="11" t="n">
         <v>0.01095759090664442</v>
       </c>
-      <c r="P9" s="10" t="n">
+      <c r="P9" s="11" t="n">
         <v>-0.0006319502785122833</v>
       </c>
-      <c r="Q9" s="10" t="n">
+      <c r="Q9" s="11" t="n">
         <v>0.01451671412948499</v>
       </c>
-      <c r="R9" s="10" t="n">
+      <c r="R9" s="11" t="n">
         <v>0.004801343554394154</v>
       </c>
-      <c r="S9" s="10" t="n">
+      <c r="S9" s="11" t="n">
         <v>-0.005835637753443541</v>
       </c>
-      <c r="T9" s="10" t="n">
+      <c r="T9" s="11" t="n">
         <v>0.01640513964927362</v>
       </c>
-      <c r="U9" s="10" t="n">
+      <c r="U9" s="11" t="n">
         <v>-0.0007653927837601216</v>
       </c>
-      <c r="V9" s="10" t="n">
+      <c r="V9" s="11" t="n">
         <v>0.01016465791095528</v>
       </c>
-      <c r="W9" s="10" t="n">
+      <c r="W9" s="11" t="n">
         <v>-0.0167544767897721</v>
       </c>
     </row>
@@ -2783,70 +3037,70 @@
           <t>中证500 (单日)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="11" t="n">
         <v>0.008954929403036351</v>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="C10" s="11" t="n">
         <v>-0.000209251312206216</v>
       </c>
-      <c r="D10" s="10" t="n">
+      <c r="D10" s="11" t="n">
         <v>0.0151702179437797</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="11" t="n">
         <v>-0.005500528171319097</v>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="11" t="n">
         <v>0.01690737109152349</v>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G10" s="11" t="n">
         <v>0.004170178500055284</v>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="H10" s="11" t="n">
         <v>0.009231398835130933</v>
       </c>
-      <c r="I10" s="10" t="n">
+      <c r="I10" s="11" t="n">
         <v>-0.002375844002544493</v>
       </c>
-      <c r="J10" s="10" t="n">
+      <c r="J10" s="11" t="n">
         <v>0.01279927687499061</v>
       </c>
-      <c r="K10" s="10" t="n">
+      <c r="K10" s="11" t="n">
         <v>-0.00966715045119367</v>
       </c>
-      <c r="L10" s="10" t="n">
+      <c r="L10" s="11" t="n">
         <v>-0.005705837117747784</v>
       </c>
-      <c r="M10" s="10" t="n">
+      <c r="M10" s="11" t="n">
         <v>0.006204348928189013</v>
       </c>
-      <c r="N10" s="10" t="n">
+      <c r="N10" s="11" t="n">
         <v>-0.01145760250156867</v>
       </c>
-      <c r="O10" s="10" t="n">
+      <c r="O10" s="11" t="n">
         <v>0.01687724908115738</v>
       </c>
-      <c r="P10" s="10" t="n">
+      <c r="P10" s="11" t="n">
         <v>0.0008494415955978729</v>
       </c>
-      <c r="Q10" s="10" t="n">
+      <c r="Q10" s="11" t="n">
         <v>0.02861627261610781</v>
       </c>
-      <c r="R10" s="10" t="n">
+      <c r="R10" s="11" t="n">
         <v>0.01261684325228851</v>
       </c>
-      <c r="S10" s="10" t="n">
+      <c r="S10" s="11" t="n">
         <v>-0.0003021801504460005</v>
       </c>
-      <c r="T10" s="10" t="n">
+      <c r="T10" s="11" t="n">
         <v>0.01674347119171547</v>
       </c>
-      <c r="U10" s="10" t="n">
+      <c r="U10" s="11" t="n">
         <v>-0.006081897304349864</v>
       </c>
-      <c r="V10" s="10" t="n">
+      <c r="V10" s="11" t="n">
         <v>0.01505351862264265</v>
       </c>
-      <c r="W10" s="10" t="n">
+      <c r="W10" s="11" t="n">
         <v>-0.02781733030478321</v>
       </c>
     </row>
@@ -2856,70 +3110,70 @@
           <t>领航1号 - 中证500 超额</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="12" t="n">
         <v>0.00954507059696365</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="12" t="n">
         <v>0.002709251312206216</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="12" t="n">
         <v>0.001329782056220299</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="12" t="n">
         <v>0.006200528171319097</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="12" t="n">
         <v>0.006392628908476512</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="12" t="n">
         <v>-0.004870178500055284</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="12" t="n">
         <v>-0.005231398835130932</v>
       </c>
-      <c r="I11" s="11" t="n">
+      <c r="I11" s="12" t="n">
         <v>0.002875844002544493</v>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="J11" s="12" t="n">
         <v>0.001200723125009384</v>
       </c>
-      <c r="K11" s="11" t="n">
+      <c r="K11" s="12" t="n">
         <v>-0.01003284954880633</v>
       </c>
-      <c r="L11" s="11" t="n">
+      <c r="L11" s="12" t="n">
         <v>0.008405837117747785</v>
       </c>
-      <c r="M11" s="11" t="n">
+      <c r="M11" s="12" t="n">
         <v>0.0009956510718109868</v>
       </c>
-      <c r="N11" s="11" t="n">
+      <c r="N11" s="12" t="n">
         <v>0.004357602501568667</v>
       </c>
-      <c r="O11" s="11" t="n">
+      <c r="O11" s="12" t="n">
         <v>0.01372275091884262</v>
       </c>
-      <c r="P11" s="11" t="n">
+      <c r="P11" s="12" t="n">
         <v>-0.0001494415955978729</v>
       </c>
-      <c r="Q11" s="11" t="n">
+      <c r="Q11" s="12" t="n">
         <v>0.01238372738389219</v>
       </c>
-      <c r="R11" s="11" t="n">
+      <c r="R11" s="12" t="n">
         <v>0.001083156747711493</v>
       </c>
-      <c r="S11" s="11" t="n">
+      <c r="S11" s="12" t="n">
         <v>-0.009297819849553999</v>
       </c>
-      <c r="T11" s="11" t="n">
+      <c r="T11" s="12" t="n">
         <v>0.009556528808284533</v>
       </c>
-      <c r="U11" s="11" t="n">
+      <c r="U11" s="12" t="n">
         <v>0.000281897304349864</v>
       </c>
-      <c r="V11" s="11" t="n">
+      <c r="V11" s="12" t="n">
         <v>0.003546481377357351</v>
       </c>
-      <c r="W11" s="11" t="n">
+      <c r="W11" s="12" t="n">
         <v>-0.002182669695216788</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Embed 领航1号 chart as PNG image so it always renders
Native openpyxl combined charts with a secondary axis are silently
dropped by some Excel/preview engines, so the user saw no chart. Render
the 领航1号 NAV (left axis) vs 领航1号-中证500 累计超额 (right axis)
plot with matplotlib and embed it as a PNG image in the 基金单位净值
sheet. Live excess formula + formula caption are unchanged.

https://claude.ai/code/session_014VmLcPuADdRYg34QDm2fTF
</commit_message>
<xml_diff>
--- a/output/20260410_20260514_table.xlsx
+++ b/output/20260410_20260514_table.xlsx
@@ -211,197 +211,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="12"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>领航1号 单位净值 与 领航1号-中证500 累计超额</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'基金单位净值'!A7</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="22000">
-              <a:solidFill>
-                <a:srgbClr val="1F6FEB"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'基金单位净值'!$B$1:$W$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'基金单位净值'!$B$7:$W$7</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'基金单位净值'!A11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="26000">
-              <a:solidFill>
-                <a:srgbClr val="9C0006"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'基金单位净值'!$B$1:$W$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'基金单位净值'!$B$11:$W$11</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="200"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>日期</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>领航1号 单位净值</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-      <valAx>
-        <axId val="200"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>领航1号-中证500 累计超额 (%)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0.00%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="max"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -409,19 +220,22 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6803999" cy="3060000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
+    <ext cx="25908000" cy="9124950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
     <clientData/>
   </oneCellAnchor>
 </wsDr>

</xml_diff>